<commit_message>
feat: Implement regional reporting functionality and update RHU encoder process guide
- Added regional reporting module to generate consolidated reports from learner records.
- Updated RHU encoder process guide to reflect changes in terminology and steps.
- Modified UI elements to include new regional reporting tab and updated instructions.
- Enhanced error handling for database schema availability checks.
- Updated requirements to include xlsxwriter for Excel report generation.
</commit_message>
<xml_diff>
--- a/programs/sbi/assets/SBI_Linelist_Template.xlsx
+++ b/programs/sbi/assets/SBI_Linelist_Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R893629171af64ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line List" sheetId="2" r:id="R47f09b0b061e4a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="3" r:id="Ra862d69401eb43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc63cc805bb804975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line List" sheetId="2" r:id="Rca0924703518437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="3" r:id="R1ed16a2b43f84554"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,6 +32,7 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
+      <x:color rgb="FF0033A0"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -136,25 +137,62 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="4">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDECEC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDECEC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDECEC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SBILinelistTable" displayName="SBILinelistTable" ref="A1:M200" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="13">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SBILearnerRecordsTable" displayName="SBILearnerRecordsTable" ref="A1:T250" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="20">
     <x:tableColumn id="1" name="Activity Date"/>
     <x:tableColumn id="2" name="School ID"/>
     <x:tableColumn id="3" name="School Name"/>
-    <x:tableColumn id="4" name="Learner ID / LRN"/>
-    <x:tableColumn id="5" name="Last Name"/>
-    <x:tableColumn id="6" name="First Name"/>
-    <x:tableColumn id="7" name="Middle Name"/>
-    <x:tableColumn id="8" name="Sex"/>
-    <x:tableColumn id="9" name="Grade Level"/>
-    <x:tableColumn id="10" name="MR Given"/>
-    <x:tableColumn id="11" name="Td Given"/>
-    <x:tableColumn id="12" name="HPV Dose"/>
-    <x:tableColumn id="13" name="Remarks"/>
+    <x:tableColumn id="4" name="Section"/>
+    <x:tableColumn id="5" name="Learner ID / LRN"/>
+    <x:tableColumn id="6" name="Last Name"/>
+    <x:tableColumn id="7" name="First Name"/>
+    <x:tableColumn id="8" name="Middle Name"/>
+    <x:tableColumn id="9" name="Sex"/>
+    <x:tableColumn id="10" name="Grade Level"/>
+    <x:tableColumn id="11" name="MR Status"/>
+    <x:tableColumn id="12" name="MR Lot/Batch No."/>
+    <x:tableColumn id="13" name="Td Status"/>
+    <x:tableColumn id="14" name="Td Lot/Batch No."/>
+    <x:tableColumn id="15" name="HPV Dose"/>
+    <x:tableColumn id="16" name="HPV Status"/>
+    <x:tableColumn id="17" name="HPV Lot/Batch No."/>
+    <x:tableColumn id="18" name="Reason Code"/>
+    <x:tableColumn id="19" name="Reason Details"/>
+    <x:tableColumn id="20" name="Remarks"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -355,13 +393,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="82" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Abra NIP Dashboard - SBI Vaccinated Learner Line List</x:v>
+        <x:v>Abra NIP Dashboard — SBI Learner Reporting Template v5.17</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -376,95 +414,87 @@
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Use one row per vaccinated learner per activity date. Upload this workbook to the Abra NIP Dashboard; the system will calculate VaccTrack totals automatically.</x:v>
+        <x:v>Use one row per learner per activity date. The dashboard calculates VaccTrack counts, regional G1/G4/G5/G7 summaries, deferrals/refusals, and reason totals.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="12" t="str">
-        <x:v>Important</x:v>
+        <x:v>Grade 1 / Grade 7</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>For a revised upload, include the COMPLETE learner list for every Activity Date + School + Grade combination present in the file. Missing existing learners in those groups will be treated as removals after confirmation.</x:v>
+        <x:v>Complete both MR Status and Td Status. Leave HPV fields blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="12" t="str">
-        <x:v>Activity Date</x:v>
+        <x:v>Grade 4 Female</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>Use the actual vaccination activity date.</x:v>
+        <x:v>Set HPV Dose to 1 or 2 and complete HPV Status. Leave MR/Td fields blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="12" t="str">
-        <x:v>School ID</x:v>
+        <x:v>Grade 5 Female</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Use the official School ID. This is the primary school matching field.</x:v>
+        <x:v>Use HPV Dose 2 only. Grade 5 is tracked for regional reporting and is NOT sent to VaccTrack.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="12" t="str">
-        <x:v>Learner ID / LRN</x:v>
+        <x:v>Statuses</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>Recommended when available. It improves duplicate and revision matching.</x:v>
+        <x:v>Use Given, Deferred, Refused, or Not Given.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="12" t="str">
-        <x:v>Names</x:v>
+        <x:v>Deferred / Refused</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>First Name and Last Name are required for the pilot. Use dummy names during dry runs.</x:v>
+        <x:v>Select one Reason Code (01–19). Reason Details is optional and is useful when Code 19 is selected.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="12" t="str">
-        <x:v>Sex</x:v>
+        <x:v>Lot / Batch</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Male or Female.</x:v>
+        <x:v>Enter the corresponding lot/batch number when a vaccine is marked Given. Blank lot/batch values are accepted but flagged for review.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="12" t="str">
-        <x:v>Grade Level</x:v>
+        <x:v>Revisions</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Grade 1, Grade 4, or Grade 7.</x:v>
+        <x:v>For a corrected upload, include the COMPLETE learner list for each Activity Date + School + Grade group in the file. Missing existing learners in those groups will be treated as removals after confirmation.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="12" t="str">
-        <x:v>MR Given / Td Given</x:v>
+        <x:v>Learner ID / LRN</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>For Grade 1 and Grade 7 only. Use Yes or No. At least one must be Yes because the sheet is for vaccinated learners.</x:v>
+        <x:v>Recommended when available because it improves duplicate and revision matching. Names are still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
-        <x:v>HPV Dose</x:v>
+        <x:v>Privacy</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>For Grade 4 only. Use 1 or 2. Grade 4 records must be Female.</x:v>
+        <x:v>This file contains identifiable vaccination information. Use authorized RHU/NIP accounts and approved handling procedures only.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
-        <x:v>Remarks</x:v>
+        <x:v>Regional clinical fields</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Optional notes. Do not enter deferral/refusal reasons here; those remain in VaccTrack.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="12" t="str">
-        <x:v>Privacy</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="str">
-        <x:v>The line list contains identifiable learner vaccination information. Use the protected RHU upload area only and avoid sharing the file outside authorized staff.</x:v>
+        <x:v>Address, date of birth, consent/allergy/sick-today screening remain on the official regional recording form; the dashboard does not collect them because they are not needed for reporting calculations.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -479,22 +509,29 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="58" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="28" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
+    <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="24" t="str">
         <x:v>Activity Date</x:v>
       </x:c>
@@ -505,39 +542,60 @@
         <x:v>School Name</x:v>
       </x:c>
       <x:c r="D1" s="24" t="str">
+        <x:v>Section</x:v>
+      </x:c>
+      <x:c r="E1" s="24" t="str">
         <x:v>Learner ID / LRN</x:v>
       </x:c>
-      <x:c r="E1" s="24" t="str">
+      <x:c r="F1" s="24" t="str">
         <x:v>Last Name</x:v>
       </x:c>
-      <x:c r="F1" s="24" t="str">
+      <x:c r="G1" s="24" t="str">
         <x:v>First Name</x:v>
       </x:c>
-      <x:c r="G1" s="24" t="str">
+      <x:c r="H1" s="24" t="str">
         <x:v>Middle Name</x:v>
       </x:c>
-      <x:c r="H1" s="24" t="str">
+      <x:c r="I1" s="24" t="str">
         <x:v>Sex</x:v>
       </x:c>
-      <x:c r="I1" s="24" t="str">
+      <x:c r="J1" s="24" t="str">
         <x:v>Grade Level</x:v>
       </x:c>
-      <x:c r="J1" s="24" t="str">
-        <x:v>MR Given</x:v>
-      </x:c>
       <x:c r="K1" s="24" t="str">
-        <x:v>Td Given</x:v>
+        <x:v>MR Status</x:v>
       </x:c>
       <x:c r="L1" s="24" t="str">
+        <x:v>MR Lot/Batch No.</x:v>
+      </x:c>
+      <x:c r="M1" s="24" t="str">
+        <x:v>Td Status</x:v>
+      </x:c>
+      <x:c r="N1" s="24" t="str">
+        <x:v>Td Lot/Batch No.</x:v>
+      </x:c>
+      <x:c r="O1" s="24" t="str">
         <x:v>HPV Dose</x:v>
       </x:c>
-      <x:c r="M1" s="24" t="str">
+      <x:c r="P1" s="24" t="str">
+        <x:v>HPV Status</x:v>
+      </x:c>
+      <x:c r="Q1" s="24" t="str">
+        <x:v>HPV Lot/Batch No.</x:v>
+      </x:c>
+      <x:c r="R1" s="24" t="str">
+        <x:v>Reason Code</x:v>
+      </x:c>
+      <x:c r="S1" s="24" t="str">
+        <x:v>Reason Details</x:v>
+      </x:c>
+      <x:c r="T1" s="24" t="str">
         <x:v>Remarks</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="30" t="n">
-        <x:v>46288</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
         <x:v>000001</x:v>
@@ -546,35 +604,48 @@
         <x:v>Sample Elementary School</x:v>
       </x:c>
       <x:c r="D2" s="16" t="str">
+        <x:v>1-A</x:v>
+      </x:c>
+      <x:c r="E2" s="16" t="str">
         <x:v>DUMMY-001</x:v>
       </x:c>
-      <x:c r="E2" s="16" t="str">
+      <x:c r="F2" s="16" t="str">
         <x:v>DELA CRUZ</x:v>
       </x:c>
-      <x:c r="F2" s="16" t="str">
+      <x:c r="G2" s="16" t="str">
         <x:v>JUAN</x:v>
       </x:c>
-      <x:c r="G2" s="16" t="str"/>
-      <x:c r="H2" s="16" t="str">
+      <x:c r="H2" s="16" t="str"/>
+      <x:c r="I2" s="16" t="str">
         <x:v>Male</x:v>
       </x:c>
-      <x:c r="I2" s="16" t="str">
+      <x:c r="J2" s="16" t="str">
         <x:v>Grade 1</x:v>
       </x:c>
-      <x:c r="J2" s="16" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
       <x:c r="K2" s="16" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="L2" s="16"/>
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="L2" s="16" t="str">
+        <x:v>MR-LOT-01</x:v>
+      </x:c>
       <x:c r="M2" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="N2" s="16" t="str">
+        <x:v>TD-LOT-01</x:v>
+      </x:c>
+      <x:c r="O2" s="16"/>
+      <x:c r="P2" s="16"/>
+      <x:c r="Q2" s="16"/>
+      <x:c r="R2" s="16"/>
+      <x:c r="S2" s="16"/>
+      <x:c r="T2" s="16" t="str">
         <x:v>DUMMY RECORD - delete before real use</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="30" t="n">
-        <x:v>46288</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
         <x:v>000001</x:v>
@@ -583,35 +654,50 @@
         <x:v>Sample Elementary School</x:v>
       </x:c>
       <x:c r="D3" s="16" t="str">
+        <x:v>1-A</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
         <x:v>DUMMY-002</x:v>
       </x:c>
-      <x:c r="E3" s="16" t="str">
+      <x:c r="F3" s="16" t="str">
         <x:v>REYES</x:v>
       </x:c>
-      <x:c r="F3" s="16" t="str">
+      <x:c r="G3" s="16" t="str">
         <x:v>MARIA</x:v>
       </x:c>
-      <x:c r="G3" s="16" t="str"/>
-      <x:c r="H3" s="16" t="str">
+      <x:c r="H3" s="16" t="str"/>
+      <x:c r="I3" s="16" t="str">
         <x:v>Female</x:v>
       </x:c>
-      <x:c r="I3" s="16" t="str">
+      <x:c r="J3" s="16" t="str">
         <x:v>Grade 1</x:v>
       </x:c>
-      <x:c r="J3" s="16" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
       <x:c r="K3" s="16" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="L3" s="16"/>
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="L3" s="16" t="str">
+        <x:v>MR-LOT-01</x:v>
+      </x:c>
       <x:c r="M3" s="16" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="N3" s="16"/>
+      <x:c r="O3" s="16"/>
+      <x:c r="P3" s="16"/>
+      <x:c r="Q3" s="16"/>
+      <x:c r="R3" s="16" t="str">
+        <x:v>11 - Child was sick, just recovered, or recently discharged from hospital</x:v>
+      </x:c>
+      <x:c r="S3" s="16" t="str">
+        <x:v>Fever today</x:v>
+      </x:c>
+      <x:c r="T3" s="16" t="str">
         <x:v>DUMMY RECORD - delete before real use</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="30" t="n">
-        <x:v>46288</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
         <x:v>000002</x:v>
@@ -620,96 +706,188 @@
         <x:v>Sample Elementary School 2</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
+        <x:v>4-A</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
         <x:v>DUMMY-003</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str">
+      <x:c r="F4" s="16" t="str">
         <x:v>SANTOS</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="str">
+      <x:c r="G4" s="16" t="str">
         <x:v>ANA</x:v>
       </x:c>
-      <x:c r="G4" s="16" t="str"/>
-      <x:c r="H4" s="16" t="str">
+      <x:c r="H4" s="16" t="str"/>
+      <x:c r="I4" s="16" t="str">
         <x:v>Female</x:v>
       </x:c>
-      <x:c r="I4" s="16" t="str">
+      <x:c r="J4" s="16" t="str">
         <x:v>Grade 4</x:v>
       </x:c>
-      <x:c r="J4" s="16"/>
       <x:c r="K4" s="16"/>
-      <x:c r="L4" s="16" t="n">
+      <x:c r="L4" s="16"/>
+      <x:c r="M4" s="16"/>
+      <x:c r="N4" s="16"/>
+      <x:c r="O4" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M4" s="16" t="str">
+      <x:c r="P4" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="Q4" s="16" t="str">
+        <x:v>HPV-LOT-01</x:v>
+      </x:c>
+      <x:c r="R4" s="16"/>
+      <x:c r="S4" s="16"/>
+      <x:c r="T4" s="16" t="str">
         <x:v>DUMMY RECORD - delete before real use</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="30" t="n">
-        <x:v>46288</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
+        <x:v>000002</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="str">
+        <x:v>Sample Elementary School 2</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="str">
+        <x:v>4-A</x:v>
+      </x:c>
+      <x:c r="E5" s="16" t="str">
+        <x:v>DUMMY-004</x:v>
+      </x:c>
+      <x:c r="F5" s="16" t="str">
+        <x:v>RAMOS</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="str">
+        <x:v>LIZA</x:v>
+      </x:c>
+      <x:c r="H5" s="16" t="str"/>
+      <x:c r="I5" s="16" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="J5" s="16" t="str">
+        <x:v>Grade 4</x:v>
+      </x:c>
+      <x:c r="K5" s="16"/>
+      <x:c r="L5" s="16"/>
+      <x:c r="M5" s="16"/>
+      <x:c r="N5" s="16"/>
+      <x:c r="O5" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P5" s="16" t="str">
+        <x:v>Refused</x:v>
+      </x:c>
+      <x:c r="Q5" s="16"/>
+      <x:c r="R5" s="16" t="str">
+        <x:v>02 - Fear of vaccine side effects</x:v>
+      </x:c>
+      <x:c r="S5" s="16"/>
+      <x:c r="T5" s="16" t="str">
+        <x:v>DUMMY RECORD - delete before real use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="30" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="str">
         <x:v>000003</x:v>
       </x:c>
-      <x:c r="C5" s="16" t="str">
-        <x:v>Sample High School</x:v>
-      </x:c>
-      <x:c r="D5" s="16" t="str">
-        <x:v>DUMMY-004</x:v>
-      </x:c>
-      <x:c r="E5" s="16" t="str">
+      <x:c r="C6" s="16" t="str">
+        <x:v>Sample Elementary School 3</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="str">
+        <x:v>5-A</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="str">
+        <x:v>DUMMY-005</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="str">
         <x:v>GARCIA</x:v>
       </x:c>
-      <x:c r="F5" s="16" t="str">
-        <x:v>PEDRO</x:v>
-      </x:c>
-      <x:c r="G5" s="16" t="str"/>
-      <x:c r="H5" s="16" t="str">
-        <x:v>Male</x:v>
-      </x:c>
-      <x:c r="I5" s="16" t="str">
-        <x:v>Grade 7</x:v>
-      </x:c>
-      <x:c r="J5" s="16" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="K5" s="16" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="L5" s="16"/>
-      <x:c r="M5" s="16" t="str">
-        <x:v>DUMMY RECORD - delete before real use</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="30"/>
-      <x:c r="B6" s="16"/>
-      <x:c r="C6" s="16"/>
-      <x:c r="D6" s="16"/>
-      <x:c r="E6" s="16"/>
-      <x:c r="F6" s="16"/>
-      <x:c r="G6" s="16"/>
-      <x:c r="H6" s="16"/>
-      <x:c r="I6" s="16"/>
-      <x:c r="J6" s="16"/>
+      <x:c r="G6" s="16" t="str">
+        <x:v>MIA</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="str"/>
+      <x:c r="I6" s="16" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="J6" s="16" t="str">
+        <x:v>Grade 5</x:v>
+      </x:c>
       <x:c r="K6" s="16"/>
       <x:c r="L6" s="16"/>
       <x:c r="M6" s="16"/>
+      <x:c r="N6" s="16"/>
+      <x:c r="O6" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P6" s="16" t="str">
+        <x:v>Not Given</x:v>
+      </x:c>
+      <x:c r="Q6" s="16"/>
+      <x:c r="R6" s="16"/>
+      <x:c r="S6" s="16" t="str">
+        <x:v>Identified without HPV Dose 2</x:v>
+      </x:c>
+      <x:c r="T6" s="16" t="str">
+        <x:v>DUMMY RECORD - regional tracking only</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30"/>
-      <x:c r="B7" s="16"/>
-      <x:c r="C7" s="16"/>
-      <x:c r="D7" s="16"/>
-      <x:c r="E7" s="16"/>
-      <x:c r="F7" s="16"/>
-      <x:c r="G7" s="16"/>
-      <x:c r="H7" s="16"/>
-      <x:c r="I7" s="16"/>
-      <x:c r="J7" s="16"/>
-      <x:c r="K7" s="16"/>
-      <x:c r="L7" s="16"/>
-      <x:c r="M7" s="16"/>
+      <x:c r="A7" s="30" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="str">
+        <x:v>000004</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="str">
+        <x:v>Sample High School</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>7-A</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="str">
+        <x:v>DUMMY-006</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="str">
+        <x:v>FLORES</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="str">
+        <x:v>PEDRO</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="str"/>
+      <x:c r="I7" s="16" t="str">
+        <x:v>Male</x:v>
+      </x:c>
+      <x:c r="J7" s="16" t="str">
+        <x:v>Grade 7</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="L7" s="16" t="str">
+        <x:v>MR-LOT-02</x:v>
+      </x:c>
+      <x:c r="M7" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="N7" s="16" t="str">
+        <x:v>TD-LOT-02</x:v>
+      </x:c>
+      <x:c r="O7" s="16"/>
+      <x:c r="P7" s="16"/>
+      <x:c r="Q7" s="16"/>
+      <x:c r="R7" s="16"/>
+      <x:c r="S7" s="16"/>
+      <x:c r="T7" s="16" t="str">
+        <x:v>DUMMY RECORD - delete before real use</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30"/>
@@ -725,6 +903,13 @@
       <x:c r="K8" s="16"/>
       <x:c r="L8" s="16"/>
       <x:c r="M8" s="16"/>
+      <x:c r="N8" s="16"/>
+      <x:c r="O8" s="16"/>
+      <x:c r="P8" s="16"/>
+      <x:c r="Q8" s="16"/>
+      <x:c r="R8" s="16"/>
+      <x:c r="S8" s="16"/>
+      <x:c r="T8" s="16"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="30"/>
@@ -740,6 +925,13 @@
       <x:c r="K9" s="16"/>
       <x:c r="L9" s="16"/>
       <x:c r="M9" s="16"/>
+      <x:c r="N9" s="16"/>
+      <x:c r="O9" s="16"/>
+      <x:c r="P9" s="16"/>
+      <x:c r="Q9" s="16"/>
+      <x:c r="R9" s="16"/>
+      <x:c r="S9" s="16"/>
+      <x:c r="T9" s="16"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="30"/>
@@ -755,6 +947,13 @@
       <x:c r="K10" s="16"/>
       <x:c r="L10" s="16"/>
       <x:c r="M10" s="16"/>
+      <x:c r="N10" s="16"/>
+      <x:c r="O10" s="16"/>
+      <x:c r="P10" s="16"/>
+      <x:c r="Q10" s="16"/>
+      <x:c r="R10" s="16"/>
+      <x:c r="S10" s="16"/>
+      <x:c r="T10" s="16"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="30"/>
@@ -770,6 +969,13 @@
       <x:c r="K11" s="16"/>
       <x:c r="L11" s="16"/>
       <x:c r="M11" s="16"/>
+      <x:c r="N11" s="16"/>
+      <x:c r="O11" s="16"/>
+      <x:c r="P11" s="16"/>
+      <x:c r="Q11" s="16"/>
+      <x:c r="R11" s="16"/>
+      <x:c r="S11" s="16"/>
+      <x:c r="T11" s="16"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="30"/>
@@ -785,6 +991,13 @@
       <x:c r="K12" s="16"/>
       <x:c r="L12" s="16"/>
       <x:c r="M12" s="16"/>
+      <x:c r="N12" s="16"/>
+      <x:c r="O12" s="16"/>
+      <x:c r="P12" s="16"/>
+      <x:c r="Q12" s="16"/>
+      <x:c r="R12" s="16"/>
+      <x:c r="S12" s="16"/>
+      <x:c r="T12" s="16"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="30"/>
@@ -800,6 +1013,13 @@
       <x:c r="K13" s="16"/>
       <x:c r="L13" s="16"/>
       <x:c r="M13" s="16"/>
+      <x:c r="N13" s="16"/>
+      <x:c r="O13" s="16"/>
+      <x:c r="P13" s="16"/>
+      <x:c r="Q13" s="16"/>
+      <x:c r="R13" s="16"/>
+      <x:c r="S13" s="16"/>
+      <x:c r="T13" s="16"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="30"/>
@@ -815,6 +1035,13 @@
       <x:c r="K14" s="16"/>
       <x:c r="L14" s="16"/>
       <x:c r="M14" s="16"/>
+      <x:c r="N14" s="16"/>
+      <x:c r="O14" s="16"/>
+      <x:c r="P14" s="16"/>
+      <x:c r="Q14" s="16"/>
+      <x:c r="R14" s="16"/>
+      <x:c r="S14" s="16"/>
+      <x:c r="T14" s="16"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="30"/>
@@ -830,6 +1057,13 @@
       <x:c r="K15" s="16"/>
       <x:c r="L15" s="16"/>
       <x:c r="M15" s="16"/>
+      <x:c r="N15" s="16"/>
+      <x:c r="O15" s="16"/>
+      <x:c r="P15" s="16"/>
+      <x:c r="Q15" s="16"/>
+      <x:c r="R15" s="16"/>
+      <x:c r="S15" s="16"/>
+      <x:c r="T15" s="16"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="30"/>
@@ -845,6 +1079,13 @@
       <x:c r="K16" s="16"/>
       <x:c r="L16" s="16"/>
       <x:c r="M16" s="16"/>
+      <x:c r="N16" s="16"/>
+      <x:c r="O16" s="16"/>
+      <x:c r="P16" s="16"/>
+      <x:c r="Q16" s="16"/>
+      <x:c r="R16" s="16"/>
+      <x:c r="S16" s="16"/>
+      <x:c r="T16" s="16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="30"/>
@@ -860,6 +1101,13 @@
       <x:c r="K17" s="16"/>
       <x:c r="L17" s="16"/>
       <x:c r="M17" s="16"/>
+      <x:c r="N17" s="16"/>
+      <x:c r="O17" s="16"/>
+      <x:c r="P17" s="16"/>
+      <x:c r="Q17" s="16"/>
+      <x:c r="R17" s="16"/>
+      <x:c r="S17" s="16"/>
+      <x:c r="T17" s="16"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30"/>
@@ -875,6 +1123,13 @@
       <x:c r="K18" s="16"/>
       <x:c r="L18" s="16"/>
       <x:c r="M18" s="16"/>
+      <x:c r="N18" s="16"/>
+      <x:c r="O18" s="16"/>
+      <x:c r="P18" s="16"/>
+      <x:c r="Q18" s="16"/>
+      <x:c r="R18" s="16"/>
+      <x:c r="S18" s="16"/>
+      <x:c r="T18" s="16"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30"/>
@@ -890,6 +1145,13 @@
       <x:c r="K19" s="16"/>
       <x:c r="L19" s="16"/>
       <x:c r="M19" s="16"/>
+      <x:c r="N19" s="16"/>
+      <x:c r="O19" s="16"/>
+      <x:c r="P19" s="16"/>
+      <x:c r="Q19" s="16"/>
+      <x:c r="R19" s="16"/>
+      <x:c r="S19" s="16"/>
+      <x:c r="T19" s="16"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="30"/>
@@ -905,6 +1167,13 @@
       <x:c r="K20" s="16"/>
       <x:c r="L20" s="16"/>
       <x:c r="M20" s="16"/>
+      <x:c r="N20" s="16"/>
+      <x:c r="O20" s="16"/>
+      <x:c r="P20" s="16"/>
+      <x:c r="Q20" s="16"/>
+      <x:c r="R20" s="16"/>
+      <x:c r="S20" s="16"/>
+      <x:c r="T20" s="16"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30"/>
@@ -920,6 +1189,13 @@
       <x:c r="K21" s="16"/>
       <x:c r="L21" s="16"/>
       <x:c r="M21" s="16"/>
+      <x:c r="N21" s="16"/>
+      <x:c r="O21" s="16"/>
+      <x:c r="P21" s="16"/>
+      <x:c r="Q21" s="16"/>
+      <x:c r="R21" s="16"/>
+      <x:c r="S21" s="16"/>
+      <x:c r="T21" s="16"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30"/>
@@ -935,6 +1211,13 @@
       <x:c r="K22" s="16"/>
       <x:c r="L22" s="16"/>
       <x:c r="M22" s="16"/>
+      <x:c r="N22" s="16"/>
+      <x:c r="O22" s="16"/>
+      <x:c r="P22" s="16"/>
+      <x:c r="Q22" s="16"/>
+      <x:c r="R22" s="16"/>
+      <x:c r="S22" s="16"/>
+      <x:c r="T22" s="16"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30"/>
@@ -950,6 +1233,13 @@
       <x:c r="K23" s="16"/>
       <x:c r="L23" s="16"/>
       <x:c r="M23" s="16"/>
+      <x:c r="N23" s="16"/>
+      <x:c r="O23" s="16"/>
+      <x:c r="P23" s="16"/>
+      <x:c r="Q23" s="16"/>
+      <x:c r="R23" s="16"/>
+      <x:c r="S23" s="16"/>
+      <x:c r="T23" s="16"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30"/>
@@ -965,6 +1255,13 @@
       <x:c r="K24" s="16"/>
       <x:c r="L24" s="16"/>
       <x:c r="M24" s="16"/>
+      <x:c r="N24" s="16"/>
+      <x:c r="O24" s="16"/>
+      <x:c r="P24" s="16"/>
+      <x:c r="Q24" s="16"/>
+      <x:c r="R24" s="16"/>
+      <x:c r="S24" s="16"/>
+      <x:c r="T24" s="16"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30"/>
@@ -980,6 +1277,13 @@
       <x:c r="K25" s="16"/>
       <x:c r="L25" s="16"/>
       <x:c r="M25" s="16"/>
+      <x:c r="N25" s="16"/>
+      <x:c r="O25" s="16"/>
+      <x:c r="P25" s="16"/>
+      <x:c r="Q25" s="16"/>
+      <x:c r="R25" s="16"/>
+      <x:c r="S25" s="16"/>
+      <x:c r="T25" s="16"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30"/>
@@ -995,6 +1299,13 @@
       <x:c r="K26" s="16"/>
       <x:c r="L26" s="16"/>
       <x:c r="M26" s="16"/>
+      <x:c r="N26" s="16"/>
+      <x:c r="O26" s="16"/>
+      <x:c r="P26" s="16"/>
+      <x:c r="Q26" s="16"/>
+      <x:c r="R26" s="16"/>
+      <x:c r="S26" s="16"/>
+      <x:c r="T26" s="16"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30"/>
@@ -1010,6 +1321,13 @@
       <x:c r="K27" s="16"/>
       <x:c r="L27" s="16"/>
       <x:c r="M27" s="16"/>
+      <x:c r="N27" s="16"/>
+      <x:c r="O27" s="16"/>
+      <x:c r="P27" s="16"/>
+      <x:c r="Q27" s="16"/>
+      <x:c r="R27" s="16"/>
+      <x:c r="S27" s="16"/>
+      <x:c r="T27" s="16"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="30"/>
@@ -1025,6 +1343,13 @@
       <x:c r="K28" s="16"/>
       <x:c r="L28" s="16"/>
       <x:c r="M28" s="16"/>
+      <x:c r="N28" s="16"/>
+      <x:c r="O28" s="16"/>
+      <x:c r="P28" s="16"/>
+      <x:c r="Q28" s="16"/>
+      <x:c r="R28" s="16"/>
+      <x:c r="S28" s="16"/>
+      <x:c r="T28" s="16"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="30"/>
@@ -1040,6 +1365,13 @@
       <x:c r="K29" s="16"/>
       <x:c r="L29" s="16"/>
       <x:c r="M29" s="16"/>
+      <x:c r="N29" s="16"/>
+      <x:c r="O29" s="16"/>
+      <x:c r="P29" s="16"/>
+      <x:c r="Q29" s="16"/>
+      <x:c r="R29" s="16"/>
+      <x:c r="S29" s="16"/>
+      <x:c r="T29" s="16"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="30"/>
@@ -1055,6 +1387,13 @@
       <x:c r="K30" s="16"/>
       <x:c r="L30" s="16"/>
       <x:c r="M30" s="16"/>
+      <x:c r="N30" s="16"/>
+      <x:c r="O30" s="16"/>
+      <x:c r="P30" s="16"/>
+      <x:c r="Q30" s="16"/>
+      <x:c r="R30" s="16"/>
+      <x:c r="S30" s="16"/>
+      <x:c r="T30" s="16"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="30"/>
@@ -1070,6 +1409,13 @@
       <x:c r="K31" s="16"/>
       <x:c r="L31" s="16"/>
       <x:c r="M31" s="16"/>
+      <x:c r="N31" s="16"/>
+      <x:c r="O31" s="16"/>
+      <x:c r="P31" s="16"/>
+      <x:c r="Q31" s="16"/>
+      <x:c r="R31" s="16"/>
+      <x:c r="S31" s="16"/>
+      <x:c r="T31" s="16"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="30"/>
@@ -1085,6 +1431,13 @@
       <x:c r="K32" s="16"/>
       <x:c r="L32" s="16"/>
       <x:c r="M32" s="16"/>
+      <x:c r="N32" s="16"/>
+      <x:c r="O32" s="16"/>
+      <x:c r="P32" s="16"/>
+      <x:c r="Q32" s="16"/>
+      <x:c r="R32" s="16"/>
+      <x:c r="S32" s="16"/>
+      <x:c r="T32" s="16"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="30"/>
@@ -1100,6 +1453,13 @@
       <x:c r="K33" s="16"/>
       <x:c r="L33" s="16"/>
       <x:c r="M33" s="16"/>
+      <x:c r="N33" s="16"/>
+      <x:c r="O33" s="16"/>
+      <x:c r="P33" s="16"/>
+      <x:c r="Q33" s="16"/>
+      <x:c r="R33" s="16"/>
+      <x:c r="S33" s="16"/>
+      <x:c r="T33" s="16"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="30"/>
@@ -1115,6 +1475,13 @@
       <x:c r="K34" s="16"/>
       <x:c r="L34" s="16"/>
       <x:c r="M34" s="16"/>
+      <x:c r="N34" s="16"/>
+      <x:c r="O34" s="16"/>
+      <x:c r="P34" s="16"/>
+      <x:c r="Q34" s="16"/>
+      <x:c r="R34" s="16"/>
+      <x:c r="S34" s="16"/>
+      <x:c r="T34" s="16"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="30"/>
@@ -1130,6 +1497,13 @@
       <x:c r="K35" s="16"/>
       <x:c r="L35" s="16"/>
       <x:c r="M35" s="16"/>
+      <x:c r="N35" s="16"/>
+      <x:c r="O35" s="16"/>
+      <x:c r="P35" s="16"/>
+      <x:c r="Q35" s="16"/>
+      <x:c r="R35" s="16"/>
+      <x:c r="S35" s="16"/>
+      <x:c r="T35" s="16"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="30"/>
@@ -1145,6 +1519,13 @@
       <x:c r="K36" s="16"/>
       <x:c r="L36" s="16"/>
       <x:c r="M36" s="16"/>
+      <x:c r="N36" s="16"/>
+      <x:c r="O36" s="16"/>
+      <x:c r="P36" s="16"/>
+      <x:c r="Q36" s="16"/>
+      <x:c r="R36" s="16"/>
+      <x:c r="S36" s="16"/>
+      <x:c r="T36" s="16"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="30"/>
@@ -1160,6 +1541,13 @@
       <x:c r="K37" s="16"/>
       <x:c r="L37" s="16"/>
       <x:c r="M37" s="16"/>
+      <x:c r="N37" s="16"/>
+      <x:c r="O37" s="16"/>
+      <x:c r="P37" s="16"/>
+      <x:c r="Q37" s="16"/>
+      <x:c r="R37" s="16"/>
+      <x:c r="S37" s="16"/>
+      <x:c r="T37" s="16"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="30"/>
@@ -1175,6 +1563,13 @@
       <x:c r="K38" s="16"/>
       <x:c r="L38" s="16"/>
       <x:c r="M38" s="16"/>
+      <x:c r="N38" s="16"/>
+      <x:c r="O38" s="16"/>
+      <x:c r="P38" s="16"/>
+      <x:c r="Q38" s="16"/>
+      <x:c r="R38" s="16"/>
+      <x:c r="S38" s="16"/>
+      <x:c r="T38" s="16"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="30"/>
@@ -1190,6 +1585,13 @@
       <x:c r="K39" s="16"/>
       <x:c r="L39" s="16"/>
       <x:c r="M39" s="16"/>
+      <x:c r="N39" s="16"/>
+      <x:c r="O39" s="16"/>
+      <x:c r="P39" s="16"/>
+      <x:c r="Q39" s="16"/>
+      <x:c r="R39" s="16"/>
+      <x:c r="S39" s="16"/>
+      <x:c r="T39" s="16"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="30"/>
@@ -1205,6 +1607,13 @@
       <x:c r="K40" s="16"/>
       <x:c r="L40" s="16"/>
       <x:c r="M40" s="16"/>
+      <x:c r="N40" s="16"/>
+      <x:c r="O40" s="16"/>
+      <x:c r="P40" s="16"/>
+      <x:c r="Q40" s="16"/>
+      <x:c r="R40" s="16"/>
+      <x:c r="S40" s="16"/>
+      <x:c r="T40" s="16"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="30"/>
@@ -1220,6 +1629,13 @@
       <x:c r="K41" s="16"/>
       <x:c r="L41" s="16"/>
       <x:c r="M41" s="16"/>
+      <x:c r="N41" s="16"/>
+      <x:c r="O41" s="16"/>
+      <x:c r="P41" s="16"/>
+      <x:c r="Q41" s="16"/>
+      <x:c r="R41" s="16"/>
+      <x:c r="S41" s="16"/>
+      <x:c r="T41" s="16"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="30"/>
@@ -1235,6 +1651,13 @@
       <x:c r="K42" s="16"/>
       <x:c r="L42" s="16"/>
       <x:c r="M42" s="16"/>
+      <x:c r="N42" s="16"/>
+      <x:c r="O42" s="16"/>
+      <x:c r="P42" s="16"/>
+      <x:c r="Q42" s="16"/>
+      <x:c r="R42" s="16"/>
+      <x:c r="S42" s="16"/>
+      <x:c r="T42" s="16"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="30"/>
@@ -1250,6 +1673,13 @@
       <x:c r="K43" s="16"/>
       <x:c r="L43" s="16"/>
       <x:c r="M43" s="16"/>
+      <x:c r="N43" s="16"/>
+      <x:c r="O43" s="16"/>
+      <x:c r="P43" s="16"/>
+      <x:c r="Q43" s="16"/>
+      <x:c r="R43" s="16"/>
+      <x:c r="S43" s="16"/>
+      <x:c r="T43" s="16"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="30"/>
@@ -1265,6 +1695,13 @@
       <x:c r="K44" s="16"/>
       <x:c r="L44" s="16"/>
       <x:c r="M44" s="16"/>
+      <x:c r="N44" s="16"/>
+      <x:c r="O44" s="16"/>
+      <x:c r="P44" s="16"/>
+      <x:c r="Q44" s="16"/>
+      <x:c r="R44" s="16"/>
+      <x:c r="S44" s="16"/>
+      <x:c r="T44" s="16"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="30"/>
@@ -1280,6 +1717,13 @@
       <x:c r="K45" s="16"/>
       <x:c r="L45" s="16"/>
       <x:c r="M45" s="16"/>
+      <x:c r="N45" s="16"/>
+      <x:c r="O45" s="16"/>
+      <x:c r="P45" s="16"/>
+      <x:c r="Q45" s="16"/>
+      <x:c r="R45" s="16"/>
+      <x:c r="S45" s="16"/>
+      <x:c r="T45" s="16"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="30"/>
@@ -1295,6 +1739,13 @@
       <x:c r="K46" s="16"/>
       <x:c r="L46" s="16"/>
       <x:c r="M46" s="16"/>
+      <x:c r="N46" s="16"/>
+      <x:c r="O46" s="16"/>
+      <x:c r="P46" s="16"/>
+      <x:c r="Q46" s="16"/>
+      <x:c r="R46" s="16"/>
+      <x:c r="S46" s="16"/>
+      <x:c r="T46" s="16"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="30"/>
@@ -1310,6 +1761,13 @@
       <x:c r="K47" s="16"/>
       <x:c r="L47" s="16"/>
       <x:c r="M47" s="16"/>
+      <x:c r="N47" s="16"/>
+      <x:c r="O47" s="16"/>
+      <x:c r="P47" s="16"/>
+      <x:c r="Q47" s="16"/>
+      <x:c r="R47" s="16"/>
+      <x:c r="S47" s="16"/>
+      <x:c r="T47" s="16"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="30"/>
@@ -1325,6 +1783,13 @@
       <x:c r="K48" s="16"/>
       <x:c r="L48" s="16"/>
       <x:c r="M48" s="16"/>
+      <x:c r="N48" s="16"/>
+      <x:c r="O48" s="16"/>
+      <x:c r="P48" s="16"/>
+      <x:c r="Q48" s="16"/>
+      <x:c r="R48" s="16"/>
+      <x:c r="S48" s="16"/>
+      <x:c r="T48" s="16"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="30"/>
@@ -1340,6 +1805,13 @@
       <x:c r="K49" s="16"/>
       <x:c r="L49" s="16"/>
       <x:c r="M49" s="16"/>
+      <x:c r="N49" s="16"/>
+      <x:c r="O49" s="16"/>
+      <x:c r="P49" s="16"/>
+      <x:c r="Q49" s="16"/>
+      <x:c r="R49" s="16"/>
+      <x:c r="S49" s="16"/>
+      <x:c r="T49" s="16"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="30"/>
@@ -1355,6 +1827,13 @@
       <x:c r="K50" s="16"/>
       <x:c r="L50" s="16"/>
       <x:c r="M50" s="16"/>
+      <x:c r="N50" s="16"/>
+      <x:c r="O50" s="16"/>
+      <x:c r="P50" s="16"/>
+      <x:c r="Q50" s="16"/>
+      <x:c r="R50" s="16"/>
+      <x:c r="S50" s="16"/>
+      <x:c r="T50" s="16"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="30"/>
@@ -1370,6 +1849,13 @@
       <x:c r="K51" s="16"/>
       <x:c r="L51" s="16"/>
       <x:c r="M51" s="16"/>
+      <x:c r="N51" s="16"/>
+      <x:c r="O51" s="16"/>
+      <x:c r="P51" s="16"/>
+      <x:c r="Q51" s="16"/>
+      <x:c r="R51" s="16"/>
+      <x:c r="S51" s="16"/>
+      <x:c r="T51" s="16"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="30"/>
@@ -1385,6 +1871,13 @@
       <x:c r="K52" s="16"/>
       <x:c r="L52" s="16"/>
       <x:c r="M52" s="16"/>
+      <x:c r="N52" s="16"/>
+      <x:c r="O52" s="16"/>
+      <x:c r="P52" s="16"/>
+      <x:c r="Q52" s="16"/>
+      <x:c r="R52" s="16"/>
+      <x:c r="S52" s="16"/>
+      <x:c r="T52" s="16"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="30"/>
@@ -1400,6 +1893,13 @@
       <x:c r="K53" s="16"/>
       <x:c r="L53" s="16"/>
       <x:c r="M53" s="16"/>
+      <x:c r="N53" s="16"/>
+      <x:c r="O53" s="16"/>
+      <x:c r="P53" s="16"/>
+      <x:c r="Q53" s="16"/>
+      <x:c r="R53" s="16"/>
+      <x:c r="S53" s="16"/>
+      <x:c r="T53" s="16"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="30"/>
@@ -1415,6 +1915,13 @@
       <x:c r="K54" s="16"/>
       <x:c r="L54" s="16"/>
       <x:c r="M54" s="16"/>
+      <x:c r="N54" s="16"/>
+      <x:c r="O54" s="16"/>
+      <x:c r="P54" s="16"/>
+      <x:c r="Q54" s="16"/>
+      <x:c r="R54" s="16"/>
+      <x:c r="S54" s="16"/>
+      <x:c r="T54" s="16"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="30"/>
@@ -1430,6 +1937,13 @@
       <x:c r="K55" s="16"/>
       <x:c r="L55" s="16"/>
       <x:c r="M55" s="16"/>
+      <x:c r="N55" s="16"/>
+      <x:c r="O55" s="16"/>
+      <x:c r="P55" s="16"/>
+      <x:c r="Q55" s="16"/>
+      <x:c r="R55" s="16"/>
+      <x:c r="S55" s="16"/>
+      <x:c r="T55" s="16"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="30"/>
@@ -1445,6 +1959,13 @@
       <x:c r="K56" s="16"/>
       <x:c r="L56" s="16"/>
       <x:c r="M56" s="16"/>
+      <x:c r="N56" s="16"/>
+      <x:c r="O56" s="16"/>
+      <x:c r="P56" s="16"/>
+      <x:c r="Q56" s="16"/>
+      <x:c r="R56" s="16"/>
+      <x:c r="S56" s="16"/>
+      <x:c r="T56" s="16"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="30"/>
@@ -1460,6 +1981,13 @@
       <x:c r="K57" s="16"/>
       <x:c r="L57" s="16"/>
       <x:c r="M57" s="16"/>
+      <x:c r="N57" s="16"/>
+      <x:c r="O57" s="16"/>
+      <x:c r="P57" s="16"/>
+      <x:c r="Q57" s="16"/>
+      <x:c r="R57" s="16"/>
+      <x:c r="S57" s="16"/>
+      <x:c r="T57" s="16"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="30"/>
@@ -1475,6 +2003,13 @@
       <x:c r="K58" s="16"/>
       <x:c r="L58" s="16"/>
       <x:c r="M58" s="16"/>
+      <x:c r="N58" s="16"/>
+      <x:c r="O58" s="16"/>
+      <x:c r="P58" s="16"/>
+      <x:c r="Q58" s="16"/>
+      <x:c r="R58" s="16"/>
+      <x:c r="S58" s="16"/>
+      <x:c r="T58" s="16"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="30"/>
@@ -1490,6 +2025,13 @@
       <x:c r="K59" s="16"/>
       <x:c r="L59" s="16"/>
       <x:c r="M59" s="16"/>
+      <x:c r="N59" s="16"/>
+      <x:c r="O59" s="16"/>
+      <x:c r="P59" s="16"/>
+      <x:c r="Q59" s="16"/>
+      <x:c r="R59" s="16"/>
+      <x:c r="S59" s="16"/>
+      <x:c r="T59" s="16"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="30"/>
@@ -1505,6 +2047,13 @@
       <x:c r="K60" s="16"/>
       <x:c r="L60" s="16"/>
       <x:c r="M60" s="16"/>
+      <x:c r="N60" s="16"/>
+      <x:c r="O60" s="16"/>
+      <x:c r="P60" s="16"/>
+      <x:c r="Q60" s="16"/>
+      <x:c r="R60" s="16"/>
+      <x:c r="S60" s="16"/>
+      <x:c r="T60" s="16"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="30"/>
@@ -1520,6 +2069,13 @@
       <x:c r="K61" s="16"/>
       <x:c r="L61" s="16"/>
       <x:c r="M61" s="16"/>
+      <x:c r="N61" s="16"/>
+      <x:c r="O61" s="16"/>
+      <x:c r="P61" s="16"/>
+      <x:c r="Q61" s="16"/>
+      <x:c r="R61" s="16"/>
+      <x:c r="S61" s="16"/>
+      <x:c r="T61" s="16"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="30"/>
@@ -1535,6 +2091,13 @@
       <x:c r="K62" s="16"/>
       <x:c r="L62" s="16"/>
       <x:c r="M62" s="16"/>
+      <x:c r="N62" s="16"/>
+      <x:c r="O62" s="16"/>
+      <x:c r="P62" s="16"/>
+      <x:c r="Q62" s="16"/>
+      <x:c r="R62" s="16"/>
+      <x:c r="S62" s="16"/>
+      <x:c r="T62" s="16"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="30"/>
@@ -1550,6 +2113,13 @@
       <x:c r="K63" s="16"/>
       <x:c r="L63" s="16"/>
       <x:c r="M63" s="16"/>
+      <x:c r="N63" s="16"/>
+      <x:c r="O63" s="16"/>
+      <x:c r="P63" s="16"/>
+      <x:c r="Q63" s="16"/>
+      <x:c r="R63" s="16"/>
+      <x:c r="S63" s="16"/>
+      <x:c r="T63" s="16"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="30"/>
@@ -1565,6 +2135,13 @@
       <x:c r="K64" s="16"/>
       <x:c r="L64" s="16"/>
       <x:c r="M64" s="16"/>
+      <x:c r="N64" s="16"/>
+      <x:c r="O64" s="16"/>
+      <x:c r="P64" s="16"/>
+      <x:c r="Q64" s="16"/>
+      <x:c r="R64" s="16"/>
+      <x:c r="S64" s="16"/>
+      <x:c r="T64" s="16"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="30"/>
@@ -1580,6 +2157,13 @@
       <x:c r="K65" s="16"/>
       <x:c r="L65" s="16"/>
       <x:c r="M65" s="16"/>
+      <x:c r="N65" s="16"/>
+      <x:c r="O65" s="16"/>
+      <x:c r="P65" s="16"/>
+      <x:c r="Q65" s="16"/>
+      <x:c r="R65" s="16"/>
+      <x:c r="S65" s="16"/>
+      <x:c r="T65" s="16"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="30"/>
@@ -1595,6 +2179,13 @@
       <x:c r="K66" s="16"/>
       <x:c r="L66" s="16"/>
       <x:c r="M66" s="16"/>
+      <x:c r="N66" s="16"/>
+      <x:c r="O66" s="16"/>
+      <x:c r="P66" s="16"/>
+      <x:c r="Q66" s="16"/>
+      <x:c r="R66" s="16"/>
+      <x:c r="S66" s="16"/>
+      <x:c r="T66" s="16"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="30"/>
@@ -1610,6 +2201,13 @@
       <x:c r="K67" s="16"/>
       <x:c r="L67" s="16"/>
       <x:c r="M67" s="16"/>
+      <x:c r="N67" s="16"/>
+      <x:c r="O67" s="16"/>
+      <x:c r="P67" s="16"/>
+      <x:c r="Q67" s="16"/>
+      <x:c r="R67" s="16"/>
+      <x:c r="S67" s="16"/>
+      <x:c r="T67" s="16"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="30"/>
@@ -1625,6 +2223,13 @@
       <x:c r="K68" s="16"/>
       <x:c r="L68" s="16"/>
       <x:c r="M68" s="16"/>
+      <x:c r="N68" s="16"/>
+      <x:c r="O68" s="16"/>
+      <x:c r="P68" s="16"/>
+      <x:c r="Q68" s="16"/>
+      <x:c r="R68" s="16"/>
+      <x:c r="S68" s="16"/>
+      <x:c r="T68" s="16"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="30"/>
@@ -1640,6 +2245,13 @@
       <x:c r="K69" s="16"/>
       <x:c r="L69" s="16"/>
       <x:c r="M69" s="16"/>
+      <x:c r="N69" s="16"/>
+      <x:c r="O69" s="16"/>
+      <x:c r="P69" s="16"/>
+      <x:c r="Q69" s="16"/>
+      <x:c r="R69" s="16"/>
+      <x:c r="S69" s="16"/>
+      <x:c r="T69" s="16"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="30"/>
@@ -1655,6 +2267,13 @@
       <x:c r="K70" s="16"/>
       <x:c r="L70" s="16"/>
       <x:c r="M70" s="16"/>
+      <x:c r="N70" s="16"/>
+      <x:c r="O70" s="16"/>
+      <x:c r="P70" s="16"/>
+      <x:c r="Q70" s="16"/>
+      <x:c r="R70" s="16"/>
+      <x:c r="S70" s="16"/>
+      <x:c r="T70" s="16"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="30"/>
@@ -1670,6 +2289,13 @@
       <x:c r="K71" s="16"/>
       <x:c r="L71" s="16"/>
       <x:c r="M71" s="16"/>
+      <x:c r="N71" s="16"/>
+      <x:c r="O71" s="16"/>
+      <x:c r="P71" s="16"/>
+      <x:c r="Q71" s="16"/>
+      <x:c r="R71" s="16"/>
+      <x:c r="S71" s="16"/>
+      <x:c r="T71" s="16"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="30"/>
@@ -1685,6 +2311,13 @@
       <x:c r="K72" s="16"/>
       <x:c r="L72" s="16"/>
       <x:c r="M72" s="16"/>
+      <x:c r="N72" s="16"/>
+      <x:c r="O72" s="16"/>
+      <x:c r="P72" s="16"/>
+      <x:c r="Q72" s="16"/>
+      <x:c r="R72" s="16"/>
+      <x:c r="S72" s="16"/>
+      <x:c r="T72" s="16"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="30"/>
@@ -1700,6 +2333,13 @@
       <x:c r="K73" s="16"/>
       <x:c r="L73" s="16"/>
       <x:c r="M73" s="16"/>
+      <x:c r="N73" s="16"/>
+      <x:c r="O73" s="16"/>
+      <x:c r="P73" s="16"/>
+      <x:c r="Q73" s="16"/>
+      <x:c r="R73" s="16"/>
+      <x:c r="S73" s="16"/>
+      <x:c r="T73" s="16"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="30"/>
@@ -1715,6 +2355,13 @@
       <x:c r="K74" s="16"/>
       <x:c r="L74" s="16"/>
       <x:c r="M74" s="16"/>
+      <x:c r="N74" s="16"/>
+      <x:c r="O74" s="16"/>
+      <x:c r="P74" s="16"/>
+      <x:c r="Q74" s="16"/>
+      <x:c r="R74" s="16"/>
+      <x:c r="S74" s="16"/>
+      <x:c r="T74" s="16"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="30"/>
@@ -1730,6 +2377,13 @@
       <x:c r="K75" s="16"/>
       <x:c r="L75" s="16"/>
       <x:c r="M75" s="16"/>
+      <x:c r="N75" s="16"/>
+      <x:c r="O75" s="16"/>
+      <x:c r="P75" s="16"/>
+      <x:c r="Q75" s="16"/>
+      <x:c r="R75" s="16"/>
+      <x:c r="S75" s="16"/>
+      <x:c r="T75" s="16"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="30"/>
@@ -1745,6 +2399,13 @@
       <x:c r="K76" s="16"/>
       <x:c r="L76" s="16"/>
       <x:c r="M76" s="16"/>
+      <x:c r="N76" s="16"/>
+      <x:c r="O76" s="16"/>
+      <x:c r="P76" s="16"/>
+      <x:c r="Q76" s="16"/>
+      <x:c r="R76" s="16"/>
+      <x:c r="S76" s="16"/>
+      <x:c r="T76" s="16"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="30"/>
@@ -1760,6 +2421,13 @@
       <x:c r="K77" s="16"/>
       <x:c r="L77" s="16"/>
       <x:c r="M77" s="16"/>
+      <x:c r="N77" s="16"/>
+      <x:c r="O77" s="16"/>
+      <x:c r="P77" s="16"/>
+      <x:c r="Q77" s="16"/>
+      <x:c r="R77" s="16"/>
+      <x:c r="S77" s="16"/>
+      <x:c r="T77" s="16"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="30"/>
@@ -1775,6 +2443,13 @@
       <x:c r="K78" s="16"/>
       <x:c r="L78" s="16"/>
       <x:c r="M78" s="16"/>
+      <x:c r="N78" s="16"/>
+      <x:c r="O78" s="16"/>
+      <x:c r="P78" s="16"/>
+      <x:c r="Q78" s="16"/>
+      <x:c r="R78" s="16"/>
+      <x:c r="S78" s="16"/>
+      <x:c r="T78" s="16"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="30"/>
@@ -1790,6 +2465,13 @@
       <x:c r="K79" s="16"/>
       <x:c r="L79" s="16"/>
       <x:c r="M79" s="16"/>
+      <x:c r="N79" s="16"/>
+      <x:c r="O79" s="16"/>
+      <x:c r="P79" s="16"/>
+      <x:c r="Q79" s="16"/>
+      <x:c r="R79" s="16"/>
+      <x:c r="S79" s="16"/>
+      <x:c r="T79" s="16"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="30"/>
@@ -1805,6 +2487,13 @@
       <x:c r="K80" s="16"/>
       <x:c r="L80" s="16"/>
       <x:c r="M80" s="16"/>
+      <x:c r="N80" s="16"/>
+      <x:c r="O80" s="16"/>
+      <x:c r="P80" s="16"/>
+      <x:c r="Q80" s="16"/>
+      <x:c r="R80" s="16"/>
+      <x:c r="S80" s="16"/>
+      <x:c r="T80" s="16"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="30"/>
@@ -1820,6 +2509,13 @@
       <x:c r="K81" s="16"/>
       <x:c r="L81" s="16"/>
       <x:c r="M81" s="16"/>
+      <x:c r="N81" s="16"/>
+      <x:c r="O81" s="16"/>
+      <x:c r="P81" s="16"/>
+      <x:c r="Q81" s="16"/>
+      <x:c r="R81" s="16"/>
+      <x:c r="S81" s="16"/>
+      <x:c r="T81" s="16"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="30"/>
@@ -1835,6 +2531,13 @@
       <x:c r="K82" s="16"/>
       <x:c r="L82" s="16"/>
       <x:c r="M82" s="16"/>
+      <x:c r="N82" s="16"/>
+      <x:c r="O82" s="16"/>
+      <x:c r="P82" s="16"/>
+      <x:c r="Q82" s="16"/>
+      <x:c r="R82" s="16"/>
+      <x:c r="S82" s="16"/>
+      <x:c r="T82" s="16"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="30"/>
@@ -1850,6 +2553,13 @@
       <x:c r="K83" s="16"/>
       <x:c r="L83" s="16"/>
       <x:c r="M83" s="16"/>
+      <x:c r="N83" s="16"/>
+      <x:c r="O83" s="16"/>
+      <x:c r="P83" s="16"/>
+      <x:c r="Q83" s="16"/>
+      <x:c r="R83" s="16"/>
+      <x:c r="S83" s="16"/>
+      <x:c r="T83" s="16"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="30"/>
@@ -1865,6 +2575,13 @@
       <x:c r="K84" s="16"/>
       <x:c r="L84" s="16"/>
       <x:c r="M84" s="16"/>
+      <x:c r="N84" s="16"/>
+      <x:c r="O84" s="16"/>
+      <x:c r="P84" s="16"/>
+      <x:c r="Q84" s="16"/>
+      <x:c r="R84" s="16"/>
+      <x:c r="S84" s="16"/>
+      <x:c r="T84" s="16"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="30"/>
@@ -1880,6 +2597,13 @@
       <x:c r="K85" s="16"/>
       <x:c r="L85" s="16"/>
       <x:c r="M85" s="16"/>
+      <x:c r="N85" s="16"/>
+      <x:c r="O85" s="16"/>
+      <x:c r="P85" s="16"/>
+      <x:c r="Q85" s="16"/>
+      <x:c r="R85" s="16"/>
+      <x:c r="S85" s="16"/>
+      <x:c r="T85" s="16"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="30"/>
@@ -1895,6 +2619,13 @@
       <x:c r="K86" s="16"/>
       <x:c r="L86" s="16"/>
       <x:c r="M86" s="16"/>
+      <x:c r="N86" s="16"/>
+      <x:c r="O86" s="16"/>
+      <x:c r="P86" s="16"/>
+      <x:c r="Q86" s="16"/>
+      <x:c r="R86" s="16"/>
+      <x:c r="S86" s="16"/>
+      <x:c r="T86" s="16"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="30"/>
@@ -1910,6 +2641,13 @@
       <x:c r="K87" s="16"/>
       <x:c r="L87" s="16"/>
       <x:c r="M87" s="16"/>
+      <x:c r="N87" s="16"/>
+      <x:c r="O87" s="16"/>
+      <x:c r="P87" s="16"/>
+      <x:c r="Q87" s="16"/>
+      <x:c r="R87" s="16"/>
+      <x:c r="S87" s="16"/>
+      <x:c r="T87" s="16"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="30"/>
@@ -1925,6 +2663,13 @@
       <x:c r="K88" s="16"/>
       <x:c r="L88" s="16"/>
       <x:c r="M88" s="16"/>
+      <x:c r="N88" s="16"/>
+      <x:c r="O88" s="16"/>
+      <x:c r="P88" s="16"/>
+      <x:c r="Q88" s="16"/>
+      <x:c r="R88" s="16"/>
+      <x:c r="S88" s="16"/>
+      <x:c r="T88" s="16"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="30"/>
@@ -1940,6 +2685,13 @@
       <x:c r="K89" s="16"/>
       <x:c r="L89" s="16"/>
       <x:c r="M89" s="16"/>
+      <x:c r="N89" s="16"/>
+      <x:c r="O89" s="16"/>
+      <x:c r="P89" s="16"/>
+      <x:c r="Q89" s="16"/>
+      <x:c r="R89" s="16"/>
+      <x:c r="S89" s="16"/>
+      <x:c r="T89" s="16"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="30"/>
@@ -1955,6 +2707,13 @@
       <x:c r="K90" s="16"/>
       <x:c r="L90" s="16"/>
       <x:c r="M90" s="16"/>
+      <x:c r="N90" s="16"/>
+      <x:c r="O90" s="16"/>
+      <x:c r="P90" s="16"/>
+      <x:c r="Q90" s="16"/>
+      <x:c r="R90" s="16"/>
+      <x:c r="S90" s="16"/>
+      <x:c r="T90" s="16"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="30"/>
@@ -1970,6 +2729,13 @@
       <x:c r="K91" s="16"/>
       <x:c r="L91" s="16"/>
       <x:c r="M91" s="16"/>
+      <x:c r="N91" s="16"/>
+      <x:c r="O91" s="16"/>
+      <x:c r="P91" s="16"/>
+      <x:c r="Q91" s="16"/>
+      <x:c r="R91" s="16"/>
+      <x:c r="S91" s="16"/>
+      <x:c r="T91" s="16"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="30"/>
@@ -1985,6 +2751,13 @@
       <x:c r="K92" s="16"/>
       <x:c r="L92" s="16"/>
       <x:c r="M92" s="16"/>
+      <x:c r="N92" s="16"/>
+      <x:c r="O92" s="16"/>
+      <x:c r="P92" s="16"/>
+      <x:c r="Q92" s="16"/>
+      <x:c r="R92" s="16"/>
+      <x:c r="S92" s="16"/>
+      <x:c r="T92" s="16"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="30"/>
@@ -2000,6 +2773,13 @@
       <x:c r="K93" s="16"/>
       <x:c r="L93" s="16"/>
       <x:c r="M93" s="16"/>
+      <x:c r="N93" s="16"/>
+      <x:c r="O93" s="16"/>
+      <x:c r="P93" s="16"/>
+      <x:c r="Q93" s="16"/>
+      <x:c r="R93" s="16"/>
+      <x:c r="S93" s="16"/>
+      <x:c r="T93" s="16"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="30"/>
@@ -2015,6 +2795,13 @@
       <x:c r="K94" s="16"/>
       <x:c r="L94" s="16"/>
       <x:c r="M94" s="16"/>
+      <x:c r="N94" s="16"/>
+      <x:c r="O94" s="16"/>
+      <x:c r="P94" s="16"/>
+      <x:c r="Q94" s="16"/>
+      <x:c r="R94" s="16"/>
+      <x:c r="S94" s="16"/>
+      <x:c r="T94" s="16"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="30"/>
@@ -2030,6 +2817,13 @@
       <x:c r="K95" s="16"/>
       <x:c r="L95" s="16"/>
       <x:c r="M95" s="16"/>
+      <x:c r="N95" s="16"/>
+      <x:c r="O95" s="16"/>
+      <x:c r="P95" s="16"/>
+      <x:c r="Q95" s="16"/>
+      <x:c r="R95" s="16"/>
+      <x:c r="S95" s="16"/>
+      <x:c r="T95" s="16"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="30"/>
@@ -2045,6 +2839,13 @@
       <x:c r="K96" s="16"/>
       <x:c r="L96" s="16"/>
       <x:c r="M96" s="16"/>
+      <x:c r="N96" s="16"/>
+      <x:c r="O96" s="16"/>
+      <x:c r="P96" s="16"/>
+      <x:c r="Q96" s="16"/>
+      <x:c r="R96" s="16"/>
+      <x:c r="S96" s="16"/>
+      <x:c r="T96" s="16"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="30"/>
@@ -2060,6 +2861,13 @@
       <x:c r="K97" s="16"/>
       <x:c r="L97" s="16"/>
       <x:c r="M97" s="16"/>
+      <x:c r="N97" s="16"/>
+      <x:c r="O97" s="16"/>
+      <x:c r="P97" s="16"/>
+      <x:c r="Q97" s="16"/>
+      <x:c r="R97" s="16"/>
+      <x:c r="S97" s="16"/>
+      <x:c r="T97" s="16"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="30"/>
@@ -2075,6 +2883,13 @@
       <x:c r="K98" s="16"/>
       <x:c r="L98" s="16"/>
       <x:c r="M98" s="16"/>
+      <x:c r="N98" s="16"/>
+      <x:c r="O98" s="16"/>
+      <x:c r="P98" s="16"/>
+      <x:c r="Q98" s="16"/>
+      <x:c r="R98" s="16"/>
+      <x:c r="S98" s="16"/>
+      <x:c r="T98" s="16"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="30"/>
@@ -2090,6 +2905,13 @@
       <x:c r="K99" s="16"/>
       <x:c r="L99" s="16"/>
       <x:c r="M99" s="16"/>
+      <x:c r="N99" s="16"/>
+      <x:c r="O99" s="16"/>
+      <x:c r="P99" s="16"/>
+      <x:c r="Q99" s="16"/>
+      <x:c r="R99" s="16"/>
+      <x:c r="S99" s="16"/>
+      <x:c r="T99" s="16"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="30"/>
@@ -2105,6 +2927,13 @@
       <x:c r="K100" s="16"/>
       <x:c r="L100" s="16"/>
       <x:c r="M100" s="16"/>
+      <x:c r="N100" s="16"/>
+      <x:c r="O100" s="16"/>
+      <x:c r="P100" s="16"/>
+      <x:c r="Q100" s="16"/>
+      <x:c r="R100" s="16"/>
+      <x:c r="S100" s="16"/>
+      <x:c r="T100" s="16"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="30"/>
@@ -2120,6 +2949,13 @@
       <x:c r="K101" s="16"/>
       <x:c r="L101" s="16"/>
       <x:c r="M101" s="16"/>
+      <x:c r="N101" s="16"/>
+      <x:c r="O101" s="16"/>
+      <x:c r="P101" s="16"/>
+      <x:c r="Q101" s="16"/>
+      <x:c r="R101" s="16"/>
+      <x:c r="S101" s="16"/>
+      <x:c r="T101" s="16"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="30"/>
@@ -2135,6 +2971,13 @@
       <x:c r="K102" s="16"/>
       <x:c r="L102" s="16"/>
       <x:c r="M102" s="16"/>
+      <x:c r="N102" s="16"/>
+      <x:c r="O102" s="16"/>
+      <x:c r="P102" s="16"/>
+      <x:c r="Q102" s="16"/>
+      <x:c r="R102" s="16"/>
+      <x:c r="S102" s="16"/>
+      <x:c r="T102" s="16"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="30"/>
@@ -2150,6 +2993,13 @@
       <x:c r="K103" s="16"/>
       <x:c r="L103" s="16"/>
       <x:c r="M103" s="16"/>
+      <x:c r="N103" s="16"/>
+      <x:c r="O103" s="16"/>
+      <x:c r="P103" s="16"/>
+      <x:c r="Q103" s="16"/>
+      <x:c r="R103" s="16"/>
+      <x:c r="S103" s="16"/>
+      <x:c r="T103" s="16"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="30"/>
@@ -2165,6 +3015,13 @@
       <x:c r="K104" s="16"/>
       <x:c r="L104" s="16"/>
       <x:c r="M104" s="16"/>
+      <x:c r="N104" s="16"/>
+      <x:c r="O104" s="16"/>
+      <x:c r="P104" s="16"/>
+      <x:c r="Q104" s="16"/>
+      <x:c r="R104" s="16"/>
+      <x:c r="S104" s="16"/>
+      <x:c r="T104" s="16"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="30"/>
@@ -2180,6 +3037,13 @@
       <x:c r="K105" s="16"/>
       <x:c r="L105" s="16"/>
       <x:c r="M105" s="16"/>
+      <x:c r="N105" s="16"/>
+      <x:c r="O105" s="16"/>
+      <x:c r="P105" s="16"/>
+      <x:c r="Q105" s="16"/>
+      <x:c r="R105" s="16"/>
+      <x:c r="S105" s="16"/>
+      <x:c r="T105" s="16"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="30"/>
@@ -2195,6 +3059,13 @@
       <x:c r="K106" s="16"/>
       <x:c r="L106" s="16"/>
       <x:c r="M106" s="16"/>
+      <x:c r="N106" s="16"/>
+      <x:c r="O106" s="16"/>
+      <x:c r="P106" s="16"/>
+      <x:c r="Q106" s="16"/>
+      <x:c r="R106" s="16"/>
+      <x:c r="S106" s="16"/>
+      <x:c r="T106" s="16"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="30"/>
@@ -2210,6 +3081,13 @@
       <x:c r="K107" s="16"/>
       <x:c r="L107" s="16"/>
       <x:c r="M107" s="16"/>
+      <x:c r="N107" s="16"/>
+      <x:c r="O107" s="16"/>
+      <x:c r="P107" s="16"/>
+      <x:c r="Q107" s="16"/>
+      <x:c r="R107" s="16"/>
+      <x:c r="S107" s="16"/>
+      <x:c r="T107" s="16"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="30"/>
@@ -2225,6 +3103,13 @@
       <x:c r="K108" s="16"/>
       <x:c r="L108" s="16"/>
       <x:c r="M108" s="16"/>
+      <x:c r="N108" s="16"/>
+      <x:c r="O108" s="16"/>
+      <x:c r="P108" s="16"/>
+      <x:c r="Q108" s="16"/>
+      <x:c r="R108" s="16"/>
+      <x:c r="S108" s="16"/>
+      <x:c r="T108" s="16"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="30"/>
@@ -2240,6 +3125,13 @@
       <x:c r="K109" s="16"/>
       <x:c r="L109" s="16"/>
       <x:c r="M109" s="16"/>
+      <x:c r="N109" s="16"/>
+      <x:c r="O109" s="16"/>
+      <x:c r="P109" s="16"/>
+      <x:c r="Q109" s="16"/>
+      <x:c r="R109" s="16"/>
+      <x:c r="S109" s="16"/>
+      <x:c r="T109" s="16"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="30"/>
@@ -2255,6 +3147,13 @@
       <x:c r="K110" s="16"/>
       <x:c r="L110" s="16"/>
       <x:c r="M110" s="16"/>
+      <x:c r="N110" s="16"/>
+      <x:c r="O110" s="16"/>
+      <x:c r="P110" s="16"/>
+      <x:c r="Q110" s="16"/>
+      <x:c r="R110" s="16"/>
+      <x:c r="S110" s="16"/>
+      <x:c r="T110" s="16"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="30"/>
@@ -2270,6 +3169,13 @@
       <x:c r="K111" s="16"/>
       <x:c r="L111" s="16"/>
       <x:c r="M111" s="16"/>
+      <x:c r="N111" s="16"/>
+      <x:c r="O111" s="16"/>
+      <x:c r="P111" s="16"/>
+      <x:c r="Q111" s="16"/>
+      <x:c r="R111" s="16"/>
+      <x:c r="S111" s="16"/>
+      <x:c r="T111" s="16"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="30"/>
@@ -2285,6 +3191,13 @@
       <x:c r="K112" s="16"/>
       <x:c r="L112" s="16"/>
       <x:c r="M112" s="16"/>
+      <x:c r="N112" s="16"/>
+      <x:c r="O112" s="16"/>
+      <x:c r="P112" s="16"/>
+      <x:c r="Q112" s="16"/>
+      <x:c r="R112" s="16"/>
+      <x:c r="S112" s="16"/>
+      <x:c r="T112" s="16"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="30"/>
@@ -2300,6 +3213,13 @@
       <x:c r="K113" s="16"/>
       <x:c r="L113" s="16"/>
       <x:c r="M113" s="16"/>
+      <x:c r="N113" s="16"/>
+      <x:c r="O113" s="16"/>
+      <x:c r="P113" s="16"/>
+      <x:c r="Q113" s="16"/>
+      <x:c r="R113" s="16"/>
+      <x:c r="S113" s="16"/>
+      <x:c r="T113" s="16"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="30"/>
@@ -2315,6 +3235,13 @@
       <x:c r="K114" s="16"/>
       <x:c r="L114" s="16"/>
       <x:c r="M114" s="16"/>
+      <x:c r="N114" s="16"/>
+      <x:c r="O114" s="16"/>
+      <x:c r="P114" s="16"/>
+      <x:c r="Q114" s="16"/>
+      <x:c r="R114" s="16"/>
+      <x:c r="S114" s="16"/>
+      <x:c r="T114" s="16"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="30"/>
@@ -2330,6 +3257,13 @@
       <x:c r="K115" s="16"/>
       <x:c r="L115" s="16"/>
       <x:c r="M115" s="16"/>
+      <x:c r="N115" s="16"/>
+      <x:c r="O115" s="16"/>
+      <x:c r="P115" s="16"/>
+      <x:c r="Q115" s="16"/>
+      <x:c r="R115" s="16"/>
+      <x:c r="S115" s="16"/>
+      <x:c r="T115" s="16"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="30"/>
@@ -2345,6 +3279,13 @@
       <x:c r="K116" s="16"/>
       <x:c r="L116" s="16"/>
       <x:c r="M116" s="16"/>
+      <x:c r="N116" s="16"/>
+      <x:c r="O116" s="16"/>
+      <x:c r="P116" s="16"/>
+      <x:c r="Q116" s="16"/>
+      <x:c r="R116" s="16"/>
+      <x:c r="S116" s="16"/>
+      <x:c r="T116" s="16"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="30"/>
@@ -2360,6 +3301,13 @@
       <x:c r="K117" s="16"/>
       <x:c r="L117" s="16"/>
       <x:c r="M117" s="16"/>
+      <x:c r="N117" s="16"/>
+      <x:c r="O117" s="16"/>
+      <x:c r="P117" s="16"/>
+      <x:c r="Q117" s="16"/>
+      <x:c r="R117" s="16"/>
+      <x:c r="S117" s="16"/>
+      <x:c r="T117" s="16"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="30"/>
@@ -2375,6 +3323,13 @@
       <x:c r="K118" s="16"/>
       <x:c r="L118" s="16"/>
       <x:c r="M118" s="16"/>
+      <x:c r="N118" s="16"/>
+      <x:c r="O118" s="16"/>
+      <x:c r="P118" s="16"/>
+      <x:c r="Q118" s="16"/>
+      <x:c r="R118" s="16"/>
+      <x:c r="S118" s="16"/>
+      <x:c r="T118" s="16"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="30"/>
@@ -2390,6 +3345,13 @@
       <x:c r="K119" s="16"/>
       <x:c r="L119" s="16"/>
       <x:c r="M119" s="16"/>
+      <x:c r="N119" s="16"/>
+      <x:c r="O119" s="16"/>
+      <x:c r="P119" s="16"/>
+      <x:c r="Q119" s="16"/>
+      <x:c r="R119" s="16"/>
+      <x:c r="S119" s="16"/>
+      <x:c r="T119" s="16"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="30"/>
@@ -2405,6 +3367,13 @@
       <x:c r="K120" s="16"/>
       <x:c r="L120" s="16"/>
       <x:c r="M120" s="16"/>
+      <x:c r="N120" s="16"/>
+      <x:c r="O120" s="16"/>
+      <x:c r="P120" s="16"/>
+      <x:c r="Q120" s="16"/>
+      <x:c r="R120" s="16"/>
+      <x:c r="S120" s="16"/>
+      <x:c r="T120" s="16"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="30"/>
@@ -2420,6 +3389,13 @@
       <x:c r="K121" s="16"/>
       <x:c r="L121" s="16"/>
       <x:c r="M121" s="16"/>
+      <x:c r="N121" s="16"/>
+      <x:c r="O121" s="16"/>
+      <x:c r="P121" s="16"/>
+      <x:c r="Q121" s="16"/>
+      <x:c r="R121" s="16"/>
+      <x:c r="S121" s="16"/>
+      <x:c r="T121" s="16"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="30"/>
@@ -2435,6 +3411,13 @@
       <x:c r="K122" s="16"/>
       <x:c r="L122" s="16"/>
       <x:c r="M122" s="16"/>
+      <x:c r="N122" s="16"/>
+      <x:c r="O122" s="16"/>
+      <x:c r="P122" s="16"/>
+      <x:c r="Q122" s="16"/>
+      <x:c r="R122" s="16"/>
+      <x:c r="S122" s="16"/>
+      <x:c r="T122" s="16"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="30"/>
@@ -2450,6 +3433,13 @@
       <x:c r="K123" s="16"/>
       <x:c r="L123" s="16"/>
       <x:c r="M123" s="16"/>
+      <x:c r="N123" s="16"/>
+      <x:c r="O123" s="16"/>
+      <x:c r="P123" s="16"/>
+      <x:c r="Q123" s="16"/>
+      <x:c r="R123" s="16"/>
+      <x:c r="S123" s="16"/>
+      <x:c r="T123" s="16"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="30"/>
@@ -2465,6 +3455,13 @@
       <x:c r="K124" s="16"/>
       <x:c r="L124" s="16"/>
       <x:c r="M124" s="16"/>
+      <x:c r="N124" s="16"/>
+      <x:c r="O124" s="16"/>
+      <x:c r="P124" s="16"/>
+      <x:c r="Q124" s="16"/>
+      <x:c r="R124" s="16"/>
+      <x:c r="S124" s="16"/>
+      <x:c r="T124" s="16"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="30"/>
@@ -2480,6 +3477,13 @@
       <x:c r="K125" s="16"/>
       <x:c r="L125" s="16"/>
       <x:c r="M125" s="16"/>
+      <x:c r="N125" s="16"/>
+      <x:c r="O125" s="16"/>
+      <x:c r="P125" s="16"/>
+      <x:c r="Q125" s="16"/>
+      <x:c r="R125" s="16"/>
+      <x:c r="S125" s="16"/>
+      <x:c r="T125" s="16"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="30"/>
@@ -2495,6 +3499,13 @@
       <x:c r="K126" s="16"/>
       <x:c r="L126" s="16"/>
       <x:c r="M126" s="16"/>
+      <x:c r="N126" s="16"/>
+      <x:c r="O126" s="16"/>
+      <x:c r="P126" s="16"/>
+      <x:c r="Q126" s="16"/>
+      <x:c r="R126" s="16"/>
+      <x:c r="S126" s="16"/>
+      <x:c r="T126" s="16"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="30"/>
@@ -2510,6 +3521,13 @@
       <x:c r="K127" s="16"/>
       <x:c r="L127" s="16"/>
       <x:c r="M127" s="16"/>
+      <x:c r="N127" s="16"/>
+      <x:c r="O127" s="16"/>
+      <x:c r="P127" s="16"/>
+      <x:c r="Q127" s="16"/>
+      <x:c r="R127" s="16"/>
+      <x:c r="S127" s="16"/>
+      <x:c r="T127" s="16"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="30"/>
@@ -2525,6 +3543,13 @@
       <x:c r="K128" s="16"/>
       <x:c r="L128" s="16"/>
       <x:c r="M128" s="16"/>
+      <x:c r="N128" s="16"/>
+      <x:c r="O128" s="16"/>
+      <x:c r="P128" s="16"/>
+      <x:c r="Q128" s="16"/>
+      <x:c r="R128" s="16"/>
+      <x:c r="S128" s="16"/>
+      <x:c r="T128" s="16"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="30"/>
@@ -2540,6 +3565,13 @@
       <x:c r="K129" s="16"/>
       <x:c r="L129" s="16"/>
       <x:c r="M129" s="16"/>
+      <x:c r="N129" s="16"/>
+      <x:c r="O129" s="16"/>
+      <x:c r="P129" s="16"/>
+      <x:c r="Q129" s="16"/>
+      <x:c r="R129" s="16"/>
+      <x:c r="S129" s="16"/>
+      <x:c r="T129" s="16"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="30"/>
@@ -2555,6 +3587,13 @@
       <x:c r="K130" s="16"/>
       <x:c r="L130" s="16"/>
       <x:c r="M130" s="16"/>
+      <x:c r="N130" s="16"/>
+      <x:c r="O130" s="16"/>
+      <x:c r="P130" s="16"/>
+      <x:c r="Q130" s="16"/>
+      <x:c r="R130" s="16"/>
+      <x:c r="S130" s="16"/>
+      <x:c r="T130" s="16"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="30"/>
@@ -2570,6 +3609,13 @@
       <x:c r="K131" s="16"/>
       <x:c r="L131" s="16"/>
       <x:c r="M131" s="16"/>
+      <x:c r="N131" s="16"/>
+      <x:c r="O131" s="16"/>
+      <x:c r="P131" s="16"/>
+      <x:c r="Q131" s="16"/>
+      <x:c r="R131" s="16"/>
+      <x:c r="S131" s="16"/>
+      <x:c r="T131" s="16"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="30"/>
@@ -2585,6 +3631,13 @@
       <x:c r="K132" s="16"/>
       <x:c r="L132" s="16"/>
       <x:c r="M132" s="16"/>
+      <x:c r="N132" s="16"/>
+      <x:c r="O132" s="16"/>
+      <x:c r="P132" s="16"/>
+      <x:c r="Q132" s="16"/>
+      <x:c r="R132" s="16"/>
+      <x:c r="S132" s="16"/>
+      <x:c r="T132" s="16"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="30"/>
@@ -2600,6 +3653,13 @@
       <x:c r="K133" s="16"/>
       <x:c r="L133" s="16"/>
       <x:c r="M133" s="16"/>
+      <x:c r="N133" s="16"/>
+      <x:c r="O133" s="16"/>
+      <x:c r="P133" s="16"/>
+      <x:c r="Q133" s="16"/>
+      <x:c r="R133" s="16"/>
+      <x:c r="S133" s="16"/>
+      <x:c r="T133" s="16"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="30"/>
@@ -2615,6 +3675,13 @@
       <x:c r="K134" s="16"/>
       <x:c r="L134" s="16"/>
       <x:c r="M134" s="16"/>
+      <x:c r="N134" s="16"/>
+      <x:c r="O134" s="16"/>
+      <x:c r="P134" s="16"/>
+      <x:c r="Q134" s="16"/>
+      <x:c r="R134" s="16"/>
+      <x:c r="S134" s="16"/>
+      <x:c r="T134" s="16"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="30"/>
@@ -2630,6 +3697,13 @@
       <x:c r="K135" s="16"/>
       <x:c r="L135" s="16"/>
       <x:c r="M135" s="16"/>
+      <x:c r="N135" s="16"/>
+      <x:c r="O135" s="16"/>
+      <x:c r="P135" s="16"/>
+      <x:c r="Q135" s="16"/>
+      <x:c r="R135" s="16"/>
+      <x:c r="S135" s="16"/>
+      <x:c r="T135" s="16"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="30"/>
@@ -2645,6 +3719,13 @@
       <x:c r="K136" s="16"/>
       <x:c r="L136" s="16"/>
       <x:c r="M136" s="16"/>
+      <x:c r="N136" s="16"/>
+      <x:c r="O136" s="16"/>
+      <x:c r="P136" s="16"/>
+      <x:c r="Q136" s="16"/>
+      <x:c r="R136" s="16"/>
+      <x:c r="S136" s="16"/>
+      <x:c r="T136" s="16"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="30"/>
@@ -2660,6 +3741,13 @@
       <x:c r="K137" s="16"/>
       <x:c r="L137" s="16"/>
       <x:c r="M137" s="16"/>
+      <x:c r="N137" s="16"/>
+      <x:c r="O137" s="16"/>
+      <x:c r="P137" s="16"/>
+      <x:c r="Q137" s="16"/>
+      <x:c r="R137" s="16"/>
+      <x:c r="S137" s="16"/>
+      <x:c r="T137" s="16"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="30"/>
@@ -2675,6 +3763,13 @@
       <x:c r="K138" s="16"/>
       <x:c r="L138" s="16"/>
       <x:c r="M138" s="16"/>
+      <x:c r="N138" s="16"/>
+      <x:c r="O138" s="16"/>
+      <x:c r="P138" s="16"/>
+      <x:c r="Q138" s="16"/>
+      <x:c r="R138" s="16"/>
+      <x:c r="S138" s="16"/>
+      <x:c r="T138" s="16"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="30"/>
@@ -2690,6 +3785,13 @@
       <x:c r="K139" s="16"/>
       <x:c r="L139" s="16"/>
       <x:c r="M139" s="16"/>
+      <x:c r="N139" s="16"/>
+      <x:c r="O139" s="16"/>
+      <x:c r="P139" s="16"/>
+      <x:c r="Q139" s="16"/>
+      <x:c r="R139" s="16"/>
+      <x:c r="S139" s="16"/>
+      <x:c r="T139" s="16"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="30"/>
@@ -2705,6 +3807,13 @@
       <x:c r="K140" s="16"/>
       <x:c r="L140" s="16"/>
       <x:c r="M140" s="16"/>
+      <x:c r="N140" s="16"/>
+      <x:c r="O140" s="16"/>
+      <x:c r="P140" s="16"/>
+      <x:c r="Q140" s="16"/>
+      <x:c r="R140" s="16"/>
+      <x:c r="S140" s="16"/>
+      <x:c r="T140" s="16"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="30"/>
@@ -2720,6 +3829,13 @@
       <x:c r="K141" s="16"/>
       <x:c r="L141" s="16"/>
       <x:c r="M141" s="16"/>
+      <x:c r="N141" s="16"/>
+      <x:c r="O141" s="16"/>
+      <x:c r="P141" s="16"/>
+      <x:c r="Q141" s="16"/>
+      <x:c r="R141" s="16"/>
+      <x:c r="S141" s="16"/>
+      <x:c r="T141" s="16"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="30"/>
@@ -2735,6 +3851,13 @@
       <x:c r="K142" s="16"/>
       <x:c r="L142" s="16"/>
       <x:c r="M142" s="16"/>
+      <x:c r="N142" s="16"/>
+      <x:c r="O142" s="16"/>
+      <x:c r="P142" s="16"/>
+      <x:c r="Q142" s="16"/>
+      <x:c r="R142" s="16"/>
+      <x:c r="S142" s="16"/>
+      <x:c r="T142" s="16"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="30"/>
@@ -2750,6 +3873,13 @@
       <x:c r="K143" s="16"/>
       <x:c r="L143" s="16"/>
       <x:c r="M143" s="16"/>
+      <x:c r="N143" s="16"/>
+      <x:c r="O143" s="16"/>
+      <x:c r="P143" s="16"/>
+      <x:c r="Q143" s="16"/>
+      <x:c r="R143" s="16"/>
+      <x:c r="S143" s="16"/>
+      <x:c r="T143" s="16"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="30"/>
@@ -2765,6 +3895,13 @@
       <x:c r="K144" s="16"/>
       <x:c r="L144" s="16"/>
       <x:c r="M144" s="16"/>
+      <x:c r="N144" s="16"/>
+      <x:c r="O144" s="16"/>
+      <x:c r="P144" s="16"/>
+      <x:c r="Q144" s="16"/>
+      <x:c r="R144" s="16"/>
+      <x:c r="S144" s="16"/>
+      <x:c r="T144" s="16"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="30"/>
@@ -2780,6 +3917,13 @@
       <x:c r="K145" s="16"/>
       <x:c r="L145" s="16"/>
       <x:c r="M145" s="16"/>
+      <x:c r="N145" s="16"/>
+      <x:c r="O145" s="16"/>
+      <x:c r="P145" s="16"/>
+      <x:c r="Q145" s="16"/>
+      <x:c r="R145" s="16"/>
+      <x:c r="S145" s="16"/>
+      <x:c r="T145" s="16"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="30"/>
@@ -2795,6 +3939,13 @@
       <x:c r="K146" s="16"/>
       <x:c r="L146" s="16"/>
       <x:c r="M146" s="16"/>
+      <x:c r="N146" s="16"/>
+      <x:c r="O146" s="16"/>
+      <x:c r="P146" s="16"/>
+      <x:c r="Q146" s="16"/>
+      <x:c r="R146" s="16"/>
+      <x:c r="S146" s="16"/>
+      <x:c r="T146" s="16"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="30"/>
@@ -2810,6 +3961,13 @@
       <x:c r="K147" s="16"/>
       <x:c r="L147" s="16"/>
       <x:c r="M147" s="16"/>
+      <x:c r="N147" s="16"/>
+      <x:c r="O147" s="16"/>
+      <x:c r="P147" s="16"/>
+      <x:c r="Q147" s="16"/>
+      <x:c r="R147" s="16"/>
+      <x:c r="S147" s="16"/>
+      <x:c r="T147" s="16"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="30"/>
@@ -2825,6 +3983,13 @@
       <x:c r="K148" s="16"/>
       <x:c r="L148" s="16"/>
       <x:c r="M148" s="16"/>
+      <x:c r="N148" s="16"/>
+      <x:c r="O148" s="16"/>
+      <x:c r="P148" s="16"/>
+      <x:c r="Q148" s="16"/>
+      <x:c r="R148" s="16"/>
+      <x:c r="S148" s="16"/>
+      <x:c r="T148" s="16"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="30"/>
@@ -2840,6 +4005,13 @@
       <x:c r="K149" s="16"/>
       <x:c r="L149" s="16"/>
       <x:c r="M149" s="16"/>
+      <x:c r="N149" s="16"/>
+      <x:c r="O149" s="16"/>
+      <x:c r="P149" s="16"/>
+      <x:c r="Q149" s="16"/>
+      <x:c r="R149" s="16"/>
+      <x:c r="S149" s="16"/>
+      <x:c r="T149" s="16"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="30"/>
@@ -2855,6 +4027,13 @@
       <x:c r="K150" s="16"/>
       <x:c r="L150" s="16"/>
       <x:c r="M150" s="16"/>
+      <x:c r="N150" s="16"/>
+      <x:c r="O150" s="16"/>
+      <x:c r="P150" s="16"/>
+      <x:c r="Q150" s="16"/>
+      <x:c r="R150" s="16"/>
+      <x:c r="S150" s="16"/>
+      <x:c r="T150" s="16"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="30"/>
@@ -2870,6 +4049,13 @@
       <x:c r="K151" s="16"/>
       <x:c r="L151" s="16"/>
       <x:c r="M151" s="16"/>
+      <x:c r="N151" s="16"/>
+      <x:c r="O151" s="16"/>
+      <x:c r="P151" s="16"/>
+      <x:c r="Q151" s="16"/>
+      <x:c r="R151" s="16"/>
+      <x:c r="S151" s="16"/>
+      <x:c r="T151" s="16"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="30"/>
@@ -2885,6 +4071,13 @@
       <x:c r="K152" s="16"/>
       <x:c r="L152" s="16"/>
       <x:c r="M152" s="16"/>
+      <x:c r="N152" s="16"/>
+      <x:c r="O152" s="16"/>
+      <x:c r="P152" s="16"/>
+      <x:c r="Q152" s="16"/>
+      <x:c r="R152" s="16"/>
+      <x:c r="S152" s="16"/>
+      <x:c r="T152" s="16"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="30"/>
@@ -2900,6 +4093,13 @@
       <x:c r="K153" s="16"/>
       <x:c r="L153" s="16"/>
       <x:c r="M153" s="16"/>
+      <x:c r="N153" s="16"/>
+      <x:c r="O153" s="16"/>
+      <x:c r="P153" s="16"/>
+      <x:c r="Q153" s="16"/>
+      <x:c r="R153" s="16"/>
+      <x:c r="S153" s="16"/>
+      <x:c r="T153" s="16"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="30"/>
@@ -2915,6 +4115,13 @@
       <x:c r="K154" s="16"/>
       <x:c r="L154" s="16"/>
       <x:c r="M154" s="16"/>
+      <x:c r="N154" s="16"/>
+      <x:c r="O154" s="16"/>
+      <x:c r="P154" s="16"/>
+      <x:c r="Q154" s="16"/>
+      <x:c r="R154" s="16"/>
+      <x:c r="S154" s="16"/>
+      <x:c r="T154" s="16"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="30"/>
@@ -2930,6 +4137,13 @@
       <x:c r="K155" s="16"/>
       <x:c r="L155" s="16"/>
       <x:c r="M155" s="16"/>
+      <x:c r="N155" s="16"/>
+      <x:c r="O155" s="16"/>
+      <x:c r="P155" s="16"/>
+      <x:c r="Q155" s="16"/>
+      <x:c r="R155" s="16"/>
+      <x:c r="S155" s="16"/>
+      <x:c r="T155" s="16"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="30"/>
@@ -2945,6 +4159,13 @@
       <x:c r="K156" s="16"/>
       <x:c r="L156" s="16"/>
       <x:c r="M156" s="16"/>
+      <x:c r="N156" s="16"/>
+      <x:c r="O156" s="16"/>
+      <x:c r="P156" s="16"/>
+      <x:c r="Q156" s="16"/>
+      <x:c r="R156" s="16"/>
+      <x:c r="S156" s="16"/>
+      <x:c r="T156" s="16"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="30"/>
@@ -2960,6 +4181,13 @@
       <x:c r="K157" s="16"/>
       <x:c r="L157" s="16"/>
       <x:c r="M157" s="16"/>
+      <x:c r="N157" s="16"/>
+      <x:c r="O157" s="16"/>
+      <x:c r="P157" s="16"/>
+      <x:c r="Q157" s="16"/>
+      <x:c r="R157" s="16"/>
+      <x:c r="S157" s="16"/>
+      <x:c r="T157" s="16"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="30"/>
@@ -2975,6 +4203,13 @@
       <x:c r="K158" s="16"/>
       <x:c r="L158" s="16"/>
       <x:c r="M158" s="16"/>
+      <x:c r="N158" s="16"/>
+      <x:c r="O158" s="16"/>
+      <x:c r="P158" s="16"/>
+      <x:c r="Q158" s="16"/>
+      <x:c r="R158" s="16"/>
+      <x:c r="S158" s="16"/>
+      <x:c r="T158" s="16"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="30"/>
@@ -2990,6 +4225,13 @@
       <x:c r="K159" s="16"/>
       <x:c r="L159" s="16"/>
       <x:c r="M159" s="16"/>
+      <x:c r="N159" s="16"/>
+      <x:c r="O159" s="16"/>
+      <x:c r="P159" s="16"/>
+      <x:c r="Q159" s="16"/>
+      <x:c r="R159" s="16"/>
+      <x:c r="S159" s="16"/>
+      <x:c r="T159" s="16"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="30"/>
@@ -3005,6 +4247,13 @@
       <x:c r="K160" s="16"/>
       <x:c r="L160" s="16"/>
       <x:c r="M160" s="16"/>
+      <x:c r="N160" s="16"/>
+      <x:c r="O160" s="16"/>
+      <x:c r="P160" s="16"/>
+      <x:c r="Q160" s="16"/>
+      <x:c r="R160" s="16"/>
+      <x:c r="S160" s="16"/>
+      <x:c r="T160" s="16"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="30"/>
@@ -3020,6 +4269,13 @@
       <x:c r="K161" s="16"/>
       <x:c r="L161" s="16"/>
       <x:c r="M161" s="16"/>
+      <x:c r="N161" s="16"/>
+      <x:c r="O161" s="16"/>
+      <x:c r="P161" s="16"/>
+      <x:c r="Q161" s="16"/>
+      <x:c r="R161" s="16"/>
+      <x:c r="S161" s="16"/>
+      <x:c r="T161" s="16"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="30"/>
@@ -3035,6 +4291,13 @@
       <x:c r="K162" s="16"/>
       <x:c r="L162" s="16"/>
       <x:c r="M162" s="16"/>
+      <x:c r="N162" s="16"/>
+      <x:c r="O162" s="16"/>
+      <x:c r="P162" s="16"/>
+      <x:c r="Q162" s="16"/>
+      <x:c r="R162" s="16"/>
+      <x:c r="S162" s="16"/>
+      <x:c r="T162" s="16"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="30"/>
@@ -3050,6 +4313,13 @@
       <x:c r="K163" s="16"/>
       <x:c r="L163" s="16"/>
       <x:c r="M163" s="16"/>
+      <x:c r="N163" s="16"/>
+      <x:c r="O163" s="16"/>
+      <x:c r="P163" s="16"/>
+      <x:c r="Q163" s="16"/>
+      <x:c r="R163" s="16"/>
+      <x:c r="S163" s="16"/>
+      <x:c r="T163" s="16"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="30"/>
@@ -3065,6 +4335,13 @@
       <x:c r="K164" s="16"/>
       <x:c r="L164" s="16"/>
       <x:c r="M164" s="16"/>
+      <x:c r="N164" s="16"/>
+      <x:c r="O164" s="16"/>
+      <x:c r="P164" s="16"/>
+      <x:c r="Q164" s="16"/>
+      <x:c r="R164" s="16"/>
+      <x:c r="S164" s="16"/>
+      <x:c r="T164" s="16"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="30"/>
@@ -3080,6 +4357,13 @@
       <x:c r="K165" s="16"/>
       <x:c r="L165" s="16"/>
       <x:c r="M165" s="16"/>
+      <x:c r="N165" s="16"/>
+      <x:c r="O165" s="16"/>
+      <x:c r="P165" s="16"/>
+      <x:c r="Q165" s="16"/>
+      <x:c r="R165" s="16"/>
+      <x:c r="S165" s="16"/>
+      <x:c r="T165" s="16"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="30"/>
@@ -3095,6 +4379,13 @@
       <x:c r="K166" s="16"/>
       <x:c r="L166" s="16"/>
       <x:c r="M166" s="16"/>
+      <x:c r="N166" s="16"/>
+      <x:c r="O166" s="16"/>
+      <x:c r="P166" s="16"/>
+      <x:c r="Q166" s="16"/>
+      <x:c r="R166" s="16"/>
+      <x:c r="S166" s="16"/>
+      <x:c r="T166" s="16"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="30"/>
@@ -3110,6 +4401,13 @@
       <x:c r="K167" s="16"/>
       <x:c r="L167" s="16"/>
       <x:c r="M167" s="16"/>
+      <x:c r="N167" s="16"/>
+      <x:c r="O167" s="16"/>
+      <x:c r="P167" s="16"/>
+      <x:c r="Q167" s="16"/>
+      <x:c r="R167" s="16"/>
+      <x:c r="S167" s="16"/>
+      <x:c r="T167" s="16"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="30"/>
@@ -3125,6 +4423,13 @@
       <x:c r="K168" s="16"/>
       <x:c r="L168" s="16"/>
       <x:c r="M168" s="16"/>
+      <x:c r="N168" s="16"/>
+      <x:c r="O168" s="16"/>
+      <x:c r="P168" s="16"/>
+      <x:c r="Q168" s="16"/>
+      <x:c r="R168" s="16"/>
+      <x:c r="S168" s="16"/>
+      <x:c r="T168" s="16"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="30"/>
@@ -3140,6 +4445,13 @@
       <x:c r="K169" s="16"/>
       <x:c r="L169" s="16"/>
       <x:c r="M169" s="16"/>
+      <x:c r="N169" s="16"/>
+      <x:c r="O169" s="16"/>
+      <x:c r="P169" s="16"/>
+      <x:c r="Q169" s="16"/>
+      <x:c r="R169" s="16"/>
+      <x:c r="S169" s="16"/>
+      <x:c r="T169" s="16"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="30"/>
@@ -3155,6 +4467,13 @@
       <x:c r="K170" s="16"/>
       <x:c r="L170" s="16"/>
       <x:c r="M170" s="16"/>
+      <x:c r="N170" s="16"/>
+      <x:c r="O170" s="16"/>
+      <x:c r="P170" s="16"/>
+      <x:c r="Q170" s="16"/>
+      <x:c r="R170" s="16"/>
+      <x:c r="S170" s="16"/>
+      <x:c r="T170" s="16"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="30"/>
@@ -3170,6 +4489,13 @@
       <x:c r="K171" s="16"/>
       <x:c r="L171" s="16"/>
       <x:c r="M171" s="16"/>
+      <x:c r="N171" s="16"/>
+      <x:c r="O171" s="16"/>
+      <x:c r="P171" s="16"/>
+      <x:c r="Q171" s="16"/>
+      <x:c r="R171" s="16"/>
+      <x:c r="S171" s="16"/>
+      <x:c r="T171" s="16"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="30"/>
@@ -3185,6 +4511,13 @@
       <x:c r="K172" s="16"/>
       <x:c r="L172" s="16"/>
       <x:c r="M172" s="16"/>
+      <x:c r="N172" s="16"/>
+      <x:c r="O172" s="16"/>
+      <x:c r="P172" s="16"/>
+      <x:c r="Q172" s="16"/>
+      <x:c r="R172" s="16"/>
+      <x:c r="S172" s="16"/>
+      <x:c r="T172" s="16"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="30"/>
@@ -3200,6 +4533,13 @@
       <x:c r="K173" s="16"/>
       <x:c r="L173" s="16"/>
       <x:c r="M173" s="16"/>
+      <x:c r="N173" s="16"/>
+      <x:c r="O173" s="16"/>
+      <x:c r="P173" s="16"/>
+      <x:c r="Q173" s="16"/>
+      <x:c r="R173" s="16"/>
+      <x:c r="S173" s="16"/>
+      <x:c r="T173" s="16"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="30"/>
@@ -3215,6 +4555,13 @@
       <x:c r="K174" s="16"/>
       <x:c r="L174" s="16"/>
       <x:c r="M174" s="16"/>
+      <x:c r="N174" s="16"/>
+      <x:c r="O174" s="16"/>
+      <x:c r="P174" s="16"/>
+      <x:c r="Q174" s="16"/>
+      <x:c r="R174" s="16"/>
+      <x:c r="S174" s="16"/>
+      <x:c r="T174" s="16"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="30"/>
@@ -3230,6 +4577,13 @@
       <x:c r="K175" s="16"/>
       <x:c r="L175" s="16"/>
       <x:c r="M175" s="16"/>
+      <x:c r="N175" s="16"/>
+      <x:c r="O175" s="16"/>
+      <x:c r="P175" s="16"/>
+      <x:c r="Q175" s="16"/>
+      <x:c r="R175" s="16"/>
+      <x:c r="S175" s="16"/>
+      <x:c r="T175" s="16"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="30"/>
@@ -3245,6 +4599,13 @@
       <x:c r="K176" s="16"/>
       <x:c r="L176" s="16"/>
       <x:c r="M176" s="16"/>
+      <x:c r="N176" s="16"/>
+      <x:c r="O176" s="16"/>
+      <x:c r="P176" s="16"/>
+      <x:c r="Q176" s="16"/>
+      <x:c r="R176" s="16"/>
+      <x:c r="S176" s="16"/>
+      <x:c r="T176" s="16"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="30"/>
@@ -3260,6 +4621,13 @@
       <x:c r="K177" s="16"/>
       <x:c r="L177" s="16"/>
       <x:c r="M177" s="16"/>
+      <x:c r="N177" s="16"/>
+      <x:c r="O177" s="16"/>
+      <x:c r="P177" s="16"/>
+      <x:c r="Q177" s="16"/>
+      <x:c r="R177" s="16"/>
+      <x:c r="S177" s="16"/>
+      <x:c r="T177" s="16"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="30"/>
@@ -3275,6 +4643,13 @@
       <x:c r="K178" s="16"/>
       <x:c r="L178" s="16"/>
       <x:c r="M178" s="16"/>
+      <x:c r="N178" s="16"/>
+      <x:c r="O178" s="16"/>
+      <x:c r="P178" s="16"/>
+      <x:c r="Q178" s="16"/>
+      <x:c r="R178" s="16"/>
+      <x:c r="S178" s="16"/>
+      <x:c r="T178" s="16"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="30"/>
@@ -3290,6 +4665,13 @@
       <x:c r="K179" s="16"/>
       <x:c r="L179" s="16"/>
       <x:c r="M179" s="16"/>
+      <x:c r="N179" s="16"/>
+      <x:c r="O179" s="16"/>
+      <x:c r="P179" s="16"/>
+      <x:c r="Q179" s="16"/>
+      <x:c r="R179" s="16"/>
+      <x:c r="S179" s="16"/>
+      <x:c r="T179" s="16"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="30"/>
@@ -3305,6 +4687,13 @@
       <x:c r="K180" s="16"/>
       <x:c r="L180" s="16"/>
       <x:c r="M180" s="16"/>
+      <x:c r="N180" s="16"/>
+      <x:c r="O180" s="16"/>
+      <x:c r="P180" s="16"/>
+      <x:c r="Q180" s="16"/>
+      <x:c r="R180" s="16"/>
+      <x:c r="S180" s="16"/>
+      <x:c r="T180" s="16"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="30"/>
@@ -3320,6 +4709,13 @@
       <x:c r="K181" s="16"/>
       <x:c r="L181" s="16"/>
       <x:c r="M181" s="16"/>
+      <x:c r="N181" s="16"/>
+      <x:c r="O181" s="16"/>
+      <x:c r="P181" s="16"/>
+      <x:c r="Q181" s="16"/>
+      <x:c r="R181" s="16"/>
+      <x:c r="S181" s="16"/>
+      <x:c r="T181" s="16"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="30"/>
@@ -3335,6 +4731,13 @@
       <x:c r="K182" s="16"/>
       <x:c r="L182" s="16"/>
       <x:c r="M182" s="16"/>
+      <x:c r="N182" s="16"/>
+      <x:c r="O182" s="16"/>
+      <x:c r="P182" s="16"/>
+      <x:c r="Q182" s="16"/>
+      <x:c r="R182" s="16"/>
+      <x:c r="S182" s="16"/>
+      <x:c r="T182" s="16"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="30"/>
@@ -3350,6 +4753,13 @@
       <x:c r="K183" s="16"/>
       <x:c r="L183" s="16"/>
       <x:c r="M183" s="16"/>
+      <x:c r="N183" s="16"/>
+      <x:c r="O183" s="16"/>
+      <x:c r="P183" s="16"/>
+      <x:c r="Q183" s="16"/>
+      <x:c r="R183" s="16"/>
+      <x:c r="S183" s="16"/>
+      <x:c r="T183" s="16"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="30"/>
@@ -3365,6 +4775,13 @@
       <x:c r="K184" s="16"/>
       <x:c r="L184" s="16"/>
       <x:c r="M184" s="16"/>
+      <x:c r="N184" s="16"/>
+      <x:c r="O184" s="16"/>
+      <x:c r="P184" s="16"/>
+      <x:c r="Q184" s="16"/>
+      <x:c r="R184" s="16"/>
+      <x:c r="S184" s="16"/>
+      <x:c r="T184" s="16"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="30"/>
@@ -3380,6 +4797,13 @@
       <x:c r="K185" s="16"/>
       <x:c r="L185" s="16"/>
       <x:c r="M185" s="16"/>
+      <x:c r="N185" s="16"/>
+      <x:c r="O185" s="16"/>
+      <x:c r="P185" s="16"/>
+      <x:c r="Q185" s="16"/>
+      <x:c r="R185" s="16"/>
+      <x:c r="S185" s="16"/>
+      <x:c r="T185" s="16"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="30"/>
@@ -3395,6 +4819,13 @@
       <x:c r="K186" s="16"/>
       <x:c r="L186" s="16"/>
       <x:c r="M186" s="16"/>
+      <x:c r="N186" s="16"/>
+      <x:c r="O186" s="16"/>
+      <x:c r="P186" s="16"/>
+      <x:c r="Q186" s="16"/>
+      <x:c r="R186" s="16"/>
+      <x:c r="S186" s="16"/>
+      <x:c r="T186" s="16"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="30"/>
@@ -3410,6 +4841,13 @@
       <x:c r="K187" s="16"/>
       <x:c r="L187" s="16"/>
       <x:c r="M187" s="16"/>
+      <x:c r="N187" s="16"/>
+      <x:c r="O187" s="16"/>
+      <x:c r="P187" s="16"/>
+      <x:c r="Q187" s="16"/>
+      <x:c r="R187" s="16"/>
+      <x:c r="S187" s="16"/>
+      <x:c r="T187" s="16"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="30"/>
@@ -3425,6 +4863,13 @@
       <x:c r="K188" s="16"/>
       <x:c r="L188" s="16"/>
       <x:c r="M188" s="16"/>
+      <x:c r="N188" s="16"/>
+      <x:c r="O188" s="16"/>
+      <x:c r="P188" s="16"/>
+      <x:c r="Q188" s="16"/>
+      <x:c r="R188" s="16"/>
+      <x:c r="S188" s="16"/>
+      <x:c r="T188" s="16"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="30"/>
@@ -3440,6 +4885,13 @@
       <x:c r="K189" s="16"/>
       <x:c r="L189" s="16"/>
       <x:c r="M189" s="16"/>
+      <x:c r="N189" s="16"/>
+      <x:c r="O189" s="16"/>
+      <x:c r="P189" s="16"/>
+      <x:c r="Q189" s="16"/>
+      <x:c r="R189" s="16"/>
+      <x:c r="S189" s="16"/>
+      <x:c r="T189" s="16"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="30"/>
@@ -3455,6 +4907,13 @@
       <x:c r="K190" s="16"/>
       <x:c r="L190" s="16"/>
       <x:c r="M190" s="16"/>
+      <x:c r="N190" s="16"/>
+      <x:c r="O190" s="16"/>
+      <x:c r="P190" s="16"/>
+      <x:c r="Q190" s="16"/>
+      <x:c r="R190" s="16"/>
+      <x:c r="S190" s="16"/>
+      <x:c r="T190" s="16"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="30"/>
@@ -3470,6 +4929,13 @@
       <x:c r="K191" s="16"/>
       <x:c r="L191" s="16"/>
       <x:c r="M191" s="16"/>
+      <x:c r="N191" s="16"/>
+      <x:c r="O191" s="16"/>
+      <x:c r="P191" s="16"/>
+      <x:c r="Q191" s="16"/>
+      <x:c r="R191" s="16"/>
+      <x:c r="S191" s="16"/>
+      <x:c r="T191" s="16"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="30"/>
@@ -3485,6 +4951,13 @@
       <x:c r="K192" s="16"/>
       <x:c r="L192" s="16"/>
       <x:c r="M192" s="16"/>
+      <x:c r="N192" s="16"/>
+      <x:c r="O192" s="16"/>
+      <x:c r="P192" s="16"/>
+      <x:c r="Q192" s="16"/>
+      <x:c r="R192" s="16"/>
+      <x:c r="S192" s="16"/>
+      <x:c r="T192" s="16"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="30"/>
@@ -3500,6 +4973,13 @@
       <x:c r="K193" s="16"/>
       <x:c r="L193" s="16"/>
       <x:c r="M193" s="16"/>
+      <x:c r="N193" s="16"/>
+      <x:c r="O193" s="16"/>
+      <x:c r="P193" s="16"/>
+      <x:c r="Q193" s="16"/>
+      <x:c r="R193" s="16"/>
+      <x:c r="S193" s="16"/>
+      <x:c r="T193" s="16"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="30"/>
@@ -3515,6 +4995,13 @@
       <x:c r="K194" s="16"/>
       <x:c r="L194" s="16"/>
       <x:c r="M194" s="16"/>
+      <x:c r="N194" s="16"/>
+      <x:c r="O194" s="16"/>
+      <x:c r="P194" s="16"/>
+      <x:c r="Q194" s="16"/>
+      <x:c r="R194" s="16"/>
+      <x:c r="S194" s="16"/>
+      <x:c r="T194" s="16"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="30"/>
@@ -3530,6 +5017,13 @@
       <x:c r="K195" s="16"/>
       <x:c r="L195" s="16"/>
       <x:c r="M195" s="16"/>
+      <x:c r="N195" s="16"/>
+      <x:c r="O195" s="16"/>
+      <x:c r="P195" s="16"/>
+      <x:c r="Q195" s="16"/>
+      <x:c r="R195" s="16"/>
+      <x:c r="S195" s="16"/>
+      <x:c r="T195" s="16"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="30"/>
@@ -3545,6 +5039,13 @@
       <x:c r="K196" s="16"/>
       <x:c r="L196" s="16"/>
       <x:c r="M196" s="16"/>
+      <x:c r="N196" s="16"/>
+      <x:c r="O196" s="16"/>
+      <x:c r="P196" s="16"/>
+      <x:c r="Q196" s="16"/>
+      <x:c r="R196" s="16"/>
+      <x:c r="S196" s="16"/>
+      <x:c r="T196" s="16"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="30"/>
@@ -3560,6 +5061,13 @@
       <x:c r="K197" s="16"/>
       <x:c r="L197" s="16"/>
       <x:c r="M197" s="16"/>
+      <x:c r="N197" s="16"/>
+      <x:c r="O197" s="16"/>
+      <x:c r="P197" s="16"/>
+      <x:c r="Q197" s="16"/>
+      <x:c r="R197" s="16"/>
+      <x:c r="S197" s="16"/>
+      <x:c r="T197" s="16"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="30"/>
@@ -3575,6 +5083,13 @@
       <x:c r="K198" s="16"/>
       <x:c r="L198" s="16"/>
       <x:c r="M198" s="16"/>
+      <x:c r="N198" s="16"/>
+      <x:c r="O198" s="16"/>
+      <x:c r="P198" s="16"/>
+      <x:c r="Q198" s="16"/>
+      <x:c r="R198" s="16"/>
+      <x:c r="S198" s="16"/>
+      <x:c r="T198" s="16"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="30"/>
@@ -3590,6 +5105,13 @@
       <x:c r="K199" s="16"/>
       <x:c r="L199" s="16"/>
       <x:c r="M199" s="16"/>
+      <x:c r="N199" s="16"/>
+      <x:c r="O199" s="16"/>
+      <x:c r="P199" s="16"/>
+      <x:c r="Q199" s="16"/>
+      <x:c r="R199" s="16"/>
+      <x:c r="S199" s="16"/>
+      <x:c r="T199" s="16"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="30"/>
@@ -3605,156 +5127,1113 @@
       <x:c r="K200" s="16"/>
       <x:c r="L200" s="16"/>
       <x:c r="M200" s="16"/>
+      <x:c r="N200" s="16"/>
+      <x:c r="O200" s="16"/>
+      <x:c r="P200" s="16"/>
+      <x:c r="Q200" s="16"/>
+      <x:c r="R200" s="16"/>
+      <x:c r="S200" s="16"/>
+      <x:c r="T200" s="16"/>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" s="28"/>
+      <x:c r="A201" s="30"/>
+      <x:c r="B201" s="16"/>
+      <x:c r="C201" s="16"/>
+      <x:c r="D201" s="16"/>
+      <x:c r="E201" s="16"/>
+      <x:c r="F201" s="16"/>
+      <x:c r="G201" s="16"/>
+      <x:c r="H201" s="16"/>
+      <x:c r="I201" s="16"/>
+      <x:c r="J201" s="16"/>
+      <x:c r="K201" s="16"/>
+      <x:c r="L201" s="16"/>
+      <x:c r="M201" s="16"/>
+      <x:c r="N201" s="16"/>
+      <x:c r="O201" s="16"/>
+      <x:c r="P201" s="16"/>
+      <x:c r="Q201" s="16"/>
+      <x:c r="R201" s="16"/>
+      <x:c r="S201" s="16"/>
+      <x:c r="T201" s="16"/>
     </x:row>
     <x:row r="202">
-      <x:c r="A202" s="28"/>
+      <x:c r="A202" s="30"/>
+      <x:c r="B202" s="16"/>
+      <x:c r="C202" s="16"/>
+      <x:c r="D202" s="16"/>
+      <x:c r="E202" s="16"/>
+      <x:c r="F202" s="16"/>
+      <x:c r="G202" s="16"/>
+      <x:c r="H202" s="16"/>
+      <x:c r="I202" s="16"/>
+      <x:c r="J202" s="16"/>
+      <x:c r="K202" s="16"/>
+      <x:c r="L202" s="16"/>
+      <x:c r="M202" s="16"/>
+      <x:c r="N202" s="16"/>
+      <x:c r="O202" s="16"/>
+      <x:c r="P202" s="16"/>
+      <x:c r="Q202" s="16"/>
+      <x:c r="R202" s="16"/>
+      <x:c r="S202" s="16"/>
+      <x:c r="T202" s="16"/>
     </x:row>
     <x:row r="203">
-      <x:c r="A203" s="28"/>
+      <x:c r="A203" s="30"/>
+      <x:c r="B203" s="16"/>
+      <x:c r="C203" s="16"/>
+      <x:c r="D203" s="16"/>
+      <x:c r="E203" s="16"/>
+      <x:c r="F203" s="16"/>
+      <x:c r="G203" s="16"/>
+      <x:c r="H203" s="16"/>
+      <x:c r="I203" s="16"/>
+      <x:c r="J203" s="16"/>
+      <x:c r="K203" s="16"/>
+      <x:c r="L203" s="16"/>
+      <x:c r="M203" s="16"/>
+      <x:c r="N203" s="16"/>
+      <x:c r="O203" s="16"/>
+      <x:c r="P203" s="16"/>
+      <x:c r="Q203" s="16"/>
+      <x:c r="R203" s="16"/>
+      <x:c r="S203" s="16"/>
+      <x:c r="T203" s="16"/>
     </x:row>
     <x:row r="204">
-      <x:c r="A204" s="28"/>
+      <x:c r="A204" s="30"/>
+      <x:c r="B204" s="16"/>
+      <x:c r="C204" s="16"/>
+      <x:c r="D204" s="16"/>
+      <x:c r="E204" s="16"/>
+      <x:c r="F204" s="16"/>
+      <x:c r="G204" s="16"/>
+      <x:c r="H204" s="16"/>
+      <x:c r="I204" s="16"/>
+      <x:c r="J204" s="16"/>
+      <x:c r="K204" s="16"/>
+      <x:c r="L204" s="16"/>
+      <x:c r="M204" s="16"/>
+      <x:c r="N204" s="16"/>
+      <x:c r="O204" s="16"/>
+      <x:c r="P204" s="16"/>
+      <x:c r="Q204" s="16"/>
+      <x:c r="R204" s="16"/>
+      <x:c r="S204" s="16"/>
+      <x:c r="T204" s="16"/>
     </x:row>
     <x:row r="205">
-      <x:c r="A205" s="28"/>
+      <x:c r="A205" s="30"/>
+      <x:c r="B205" s="16"/>
+      <x:c r="C205" s="16"/>
+      <x:c r="D205" s="16"/>
+      <x:c r="E205" s="16"/>
+      <x:c r="F205" s="16"/>
+      <x:c r="G205" s="16"/>
+      <x:c r="H205" s="16"/>
+      <x:c r="I205" s="16"/>
+      <x:c r="J205" s="16"/>
+      <x:c r="K205" s="16"/>
+      <x:c r="L205" s="16"/>
+      <x:c r="M205" s="16"/>
+      <x:c r="N205" s="16"/>
+      <x:c r="O205" s="16"/>
+      <x:c r="P205" s="16"/>
+      <x:c r="Q205" s="16"/>
+      <x:c r="R205" s="16"/>
+      <x:c r="S205" s="16"/>
+      <x:c r="T205" s="16"/>
     </x:row>
     <x:row r="206">
-      <x:c r="A206" s="28"/>
+      <x:c r="A206" s="30"/>
+      <x:c r="B206" s="16"/>
+      <x:c r="C206" s="16"/>
+      <x:c r="D206" s="16"/>
+      <x:c r="E206" s="16"/>
+      <x:c r="F206" s="16"/>
+      <x:c r="G206" s="16"/>
+      <x:c r="H206" s="16"/>
+      <x:c r="I206" s="16"/>
+      <x:c r="J206" s="16"/>
+      <x:c r="K206" s="16"/>
+      <x:c r="L206" s="16"/>
+      <x:c r="M206" s="16"/>
+      <x:c r="N206" s="16"/>
+      <x:c r="O206" s="16"/>
+      <x:c r="P206" s="16"/>
+      <x:c r="Q206" s="16"/>
+      <x:c r="R206" s="16"/>
+      <x:c r="S206" s="16"/>
+      <x:c r="T206" s="16"/>
     </x:row>
     <x:row r="207">
-      <x:c r="A207" s="28"/>
+      <x:c r="A207" s="30"/>
+      <x:c r="B207" s="16"/>
+      <x:c r="C207" s="16"/>
+      <x:c r="D207" s="16"/>
+      <x:c r="E207" s="16"/>
+      <x:c r="F207" s="16"/>
+      <x:c r="G207" s="16"/>
+      <x:c r="H207" s="16"/>
+      <x:c r="I207" s="16"/>
+      <x:c r="J207" s="16"/>
+      <x:c r="K207" s="16"/>
+      <x:c r="L207" s="16"/>
+      <x:c r="M207" s="16"/>
+      <x:c r="N207" s="16"/>
+      <x:c r="O207" s="16"/>
+      <x:c r="P207" s="16"/>
+      <x:c r="Q207" s="16"/>
+      <x:c r="R207" s="16"/>
+      <x:c r="S207" s="16"/>
+      <x:c r="T207" s="16"/>
     </x:row>
     <x:row r="208">
-      <x:c r="A208" s="28"/>
+      <x:c r="A208" s="30"/>
+      <x:c r="B208" s="16"/>
+      <x:c r="C208" s="16"/>
+      <x:c r="D208" s="16"/>
+      <x:c r="E208" s="16"/>
+      <x:c r="F208" s="16"/>
+      <x:c r="G208" s="16"/>
+      <x:c r="H208" s="16"/>
+      <x:c r="I208" s="16"/>
+      <x:c r="J208" s="16"/>
+      <x:c r="K208" s="16"/>
+      <x:c r="L208" s="16"/>
+      <x:c r="M208" s="16"/>
+      <x:c r="N208" s="16"/>
+      <x:c r="O208" s="16"/>
+      <x:c r="P208" s="16"/>
+      <x:c r="Q208" s="16"/>
+      <x:c r="R208" s="16"/>
+      <x:c r="S208" s="16"/>
+      <x:c r="T208" s="16"/>
     </x:row>
     <x:row r="209">
-      <x:c r="A209" s="28"/>
+      <x:c r="A209" s="30"/>
+      <x:c r="B209" s="16"/>
+      <x:c r="C209" s="16"/>
+      <x:c r="D209" s="16"/>
+      <x:c r="E209" s="16"/>
+      <x:c r="F209" s="16"/>
+      <x:c r="G209" s="16"/>
+      <x:c r="H209" s="16"/>
+      <x:c r="I209" s="16"/>
+      <x:c r="J209" s="16"/>
+      <x:c r="K209" s="16"/>
+      <x:c r="L209" s="16"/>
+      <x:c r="M209" s="16"/>
+      <x:c r="N209" s="16"/>
+      <x:c r="O209" s="16"/>
+      <x:c r="P209" s="16"/>
+      <x:c r="Q209" s="16"/>
+      <x:c r="R209" s="16"/>
+      <x:c r="S209" s="16"/>
+      <x:c r="T209" s="16"/>
     </x:row>
     <x:row r="210">
-      <x:c r="A210" s="28"/>
+      <x:c r="A210" s="30"/>
+      <x:c r="B210" s="16"/>
+      <x:c r="C210" s="16"/>
+      <x:c r="D210" s="16"/>
+      <x:c r="E210" s="16"/>
+      <x:c r="F210" s="16"/>
+      <x:c r="G210" s="16"/>
+      <x:c r="H210" s="16"/>
+      <x:c r="I210" s="16"/>
+      <x:c r="J210" s="16"/>
+      <x:c r="K210" s="16"/>
+      <x:c r="L210" s="16"/>
+      <x:c r="M210" s="16"/>
+      <x:c r="N210" s="16"/>
+      <x:c r="O210" s="16"/>
+      <x:c r="P210" s="16"/>
+      <x:c r="Q210" s="16"/>
+      <x:c r="R210" s="16"/>
+      <x:c r="S210" s="16"/>
+      <x:c r="T210" s="16"/>
     </x:row>
     <x:row r="211">
-      <x:c r="A211" s="28"/>
+      <x:c r="A211" s="30"/>
+      <x:c r="B211" s="16"/>
+      <x:c r="C211" s="16"/>
+      <x:c r="D211" s="16"/>
+      <x:c r="E211" s="16"/>
+      <x:c r="F211" s="16"/>
+      <x:c r="G211" s="16"/>
+      <x:c r="H211" s="16"/>
+      <x:c r="I211" s="16"/>
+      <x:c r="J211" s="16"/>
+      <x:c r="K211" s="16"/>
+      <x:c r="L211" s="16"/>
+      <x:c r="M211" s="16"/>
+      <x:c r="N211" s="16"/>
+      <x:c r="O211" s="16"/>
+      <x:c r="P211" s="16"/>
+      <x:c r="Q211" s="16"/>
+      <x:c r="R211" s="16"/>
+      <x:c r="S211" s="16"/>
+      <x:c r="T211" s="16"/>
     </x:row>
     <x:row r="212">
-      <x:c r="A212" s="28"/>
+      <x:c r="A212" s="30"/>
+      <x:c r="B212" s="16"/>
+      <x:c r="C212" s="16"/>
+      <x:c r="D212" s="16"/>
+      <x:c r="E212" s="16"/>
+      <x:c r="F212" s="16"/>
+      <x:c r="G212" s="16"/>
+      <x:c r="H212" s="16"/>
+      <x:c r="I212" s="16"/>
+      <x:c r="J212" s="16"/>
+      <x:c r="K212" s="16"/>
+      <x:c r="L212" s="16"/>
+      <x:c r="M212" s="16"/>
+      <x:c r="N212" s="16"/>
+      <x:c r="O212" s="16"/>
+      <x:c r="P212" s="16"/>
+      <x:c r="Q212" s="16"/>
+      <x:c r="R212" s="16"/>
+      <x:c r="S212" s="16"/>
+      <x:c r="T212" s="16"/>
     </x:row>
     <x:row r="213">
-      <x:c r="A213" s="28"/>
+      <x:c r="A213" s="30"/>
+      <x:c r="B213" s="16"/>
+      <x:c r="C213" s="16"/>
+      <x:c r="D213" s="16"/>
+      <x:c r="E213" s="16"/>
+      <x:c r="F213" s="16"/>
+      <x:c r="G213" s="16"/>
+      <x:c r="H213" s="16"/>
+      <x:c r="I213" s="16"/>
+      <x:c r="J213" s="16"/>
+      <x:c r="K213" s="16"/>
+      <x:c r="L213" s="16"/>
+      <x:c r="M213" s="16"/>
+      <x:c r="N213" s="16"/>
+      <x:c r="O213" s="16"/>
+      <x:c r="P213" s="16"/>
+      <x:c r="Q213" s="16"/>
+      <x:c r="R213" s="16"/>
+      <x:c r="S213" s="16"/>
+      <x:c r="T213" s="16"/>
     </x:row>
     <x:row r="214">
-      <x:c r="A214" s="28"/>
+      <x:c r="A214" s="30"/>
+      <x:c r="B214" s="16"/>
+      <x:c r="C214" s="16"/>
+      <x:c r="D214" s="16"/>
+      <x:c r="E214" s="16"/>
+      <x:c r="F214" s="16"/>
+      <x:c r="G214" s="16"/>
+      <x:c r="H214" s="16"/>
+      <x:c r="I214" s="16"/>
+      <x:c r="J214" s="16"/>
+      <x:c r="K214" s="16"/>
+      <x:c r="L214" s="16"/>
+      <x:c r="M214" s="16"/>
+      <x:c r="N214" s="16"/>
+      <x:c r="O214" s="16"/>
+      <x:c r="P214" s="16"/>
+      <x:c r="Q214" s="16"/>
+      <x:c r="R214" s="16"/>
+      <x:c r="S214" s="16"/>
+      <x:c r="T214" s="16"/>
     </x:row>
     <x:row r="215">
-      <x:c r="A215" s="28"/>
+      <x:c r="A215" s="30"/>
+      <x:c r="B215" s="16"/>
+      <x:c r="C215" s="16"/>
+      <x:c r="D215" s="16"/>
+      <x:c r="E215" s="16"/>
+      <x:c r="F215" s="16"/>
+      <x:c r="G215" s="16"/>
+      <x:c r="H215" s="16"/>
+      <x:c r="I215" s="16"/>
+      <x:c r="J215" s="16"/>
+      <x:c r="K215" s="16"/>
+      <x:c r="L215" s="16"/>
+      <x:c r="M215" s="16"/>
+      <x:c r="N215" s="16"/>
+      <x:c r="O215" s="16"/>
+      <x:c r="P215" s="16"/>
+      <x:c r="Q215" s="16"/>
+      <x:c r="R215" s="16"/>
+      <x:c r="S215" s="16"/>
+      <x:c r="T215" s="16"/>
     </x:row>
     <x:row r="216">
-      <x:c r="A216" s="28"/>
+      <x:c r="A216" s="30"/>
+      <x:c r="B216" s="16"/>
+      <x:c r="C216" s="16"/>
+      <x:c r="D216" s="16"/>
+      <x:c r="E216" s="16"/>
+      <x:c r="F216" s="16"/>
+      <x:c r="G216" s="16"/>
+      <x:c r="H216" s="16"/>
+      <x:c r="I216" s="16"/>
+      <x:c r="J216" s="16"/>
+      <x:c r="K216" s="16"/>
+      <x:c r="L216" s="16"/>
+      <x:c r="M216" s="16"/>
+      <x:c r="N216" s="16"/>
+      <x:c r="O216" s="16"/>
+      <x:c r="P216" s="16"/>
+      <x:c r="Q216" s="16"/>
+      <x:c r="R216" s="16"/>
+      <x:c r="S216" s="16"/>
+      <x:c r="T216" s="16"/>
     </x:row>
     <x:row r="217">
-      <x:c r="A217" s="28"/>
+      <x:c r="A217" s="30"/>
+      <x:c r="B217" s="16"/>
+      <x:c r="C217" s="16"/>
+      <x:c r="D217" s="16"/>
+      <x:c r="E217" s="16"/>
+      <x:c r="F217" s="16"/>
+      <x:c r="G217" s="16"/>
+      <x:c r="H217" s="16"/>
+      <x:c r="I217" s="16"/>
+      <x:c r="J217" s="16"/>
+      <x:c r="K217" s="16"/>
+      <x:c r="L217" s="16"/>
+      <x:c r="M217" s="16"/>
+      <x:c r="N217" s="16"/>
+      <x:c r="O217" s="16"/>
+      <x:c r="P217" s="16"/>
+      <x:c r="Q217" s="16"/>
+      <x:c r="R217" s="16"/>
+      <x:c r="S217" s="16"/>
+      <x:c r="T217" s="16"/>
     </x:row>
     <x:row r="218">
-      <x:c r="A218" s="28"/>
+      <x:c r="A218" s="30"/>
+      <x:c r="B218" s="16"/>
+      <x:c r="C218" s="16"/>
+      <x:c r="D218" s="16"/>
+      <x:c r="E218" s="16"/>
+      <x:c r="F218" s="16"/>
+      <x:c r="G218" s="16"/>
+      <x:c r="H218" s="16"/>
+      <x:c r="I218" s="16"/>
+      <x:c r="J218" s="16"/>
+      <x:c r="K218" s="16"/>
+      <x:c r="L218" s="16"/>
+      <x:c r="M218" s="16"/>
+      <x:c r="N218" s="16"/>
+      <x:c r="O218" s="16"/>
+      <x:c r="P218" s="16"/>
+      <x:c r="Q218" s="16"/>
+      <x:c r="R218" s="16"/>
+      <x:c r="S218" s="16"/>
+      <x:c r="T218" s="16"/>
     </x:row>
     <x:row r="219">
-      <x:c r="A219" s="28"/>
+      <x:c r="A219" s="30"/>
+      <x:c r="B219" s="16"/>
+      <x:c r="C219" s="16"/>
+      <x:c r="D219" s="16"/>
+      <x:c r="E219" s="16"/>
+      <x:c r="F219" s="16"/>
+      <x:c r="G219" s="16"/>
+      <x:c r="H219" s="16"/>
+      <x:c r="I219" s="16"/>
+      <x:c r="J219" s="16"/>
+      <x:c r="K219" s="16"/>
+      <x:c r="L219" s="16"/>
+      <x:c r="M219" s="16"/>
+      <x:c r="N219" s="16"/>
+      <x:c r="O219" s="16"/>
+      <x:c r="P219" s="16"/>
+      <x:c r="Q219" s="16"/>
+      <x:c r="R219" s="16"/>
+      <x:c r="S219" s="16"/>
+      <x:c r="T219" s="16"/>
     </x:row>
     <x:row r="220">
-      <x:c r="A220" s="28"/>
+      <x:c r="A220" s="30"/>
+      <x:c r="B220" s="16"/>
+      <x:c r="C220" s="16"/>
+      <x:c r="D220" s="16"/>
+      <x:c r="E220" s="16"/>
+      <x:c r="F220" s="16"/>
+      <x:c r="G220" s="16"/>
+      <x:c r="H220" s="16"/>
+      <x:c r="I220" s="16"/>
+      <x:c r="J220" s="16"/>
+      <x:c r="K220" s="16"/>
+      <x:c r="L220" s="16"/>
+      <x:c r="M220" s="16"/>
+      <x:c r="N220" s="16"/>
+      <x:c r="O220" s="16"/>
+      <x:c r="P220" s="16"/>
+      <x:c r="Q220" s="16"/>
+      <x:c r="R220" s="16"/>
+      <x:c r="S220" s="16"/>
+      <x:c r="T220" s="16"/>
     </x:row>
     <x:row r="221">
-      <x:c r="A221" s="28"/>
+      <x:c r="A221" s="30"/>
+      <x:c r="B221" s="16"/>
+      <x:c r="C221" s="16"/>
+      <x:c r="D221" s="16"/>
+      <x:c r="E221" s="16"/>
+      <x:c r="F221" s="16"/>
+      <x:c r="G221" s="16"/>
+      <x:c r="H221" s="16"/>
+      <x:c r="I221" s="16"/>
+      <x:c r="J221" s="16"/>
+      <x:c r="K221" s="16"/>
+      <x:c r="L221" s="16"/>
+      <x:c r="M221" s="16"/>
+      <x:c r="N221" s="16"/>
+      <x:c r="O221" s="16"/>
+      <x:c r="P221" s="16"/>
+      <x:c r="Q221" s="16"/>
+      <x:c r="R221" s="16"/>
+      <x:c r="S221" s="16"/>
+      <x:c r="T221" s="16"/>
     </x:row>
     <x:row r="222">
-      <x:c r="A222" s="28"/>
+      <x:c r="A222" s="30"/>
+      <x:c r="B222" s="16"/>
+      <x:c r="C222" s="16"/>
+      <x:c r="D222" s="16"/>
+      <x:c r="E222" s="16"/>
+      <x:c r="F222" s="16"/>
+      <x:c r="G222" s="16"/>
+      <x:c r="H222" s="16"/>
+      <x:c r="I222" s="16"/>
+      <x:c r="J222" s="16"/>
+      <x:c r="K222" s="16"/>
+      <x:c r="L222" s="16"/>
+      <x:c r="M222" s="16"/>
+      <x:c r="N222" s="16"/>
+      <x:c r="O222" s="16"/>
+      <x:c r="P222" s="16"/>
+      <x:c r="Q222" s="16"/>
+      <x:c r="R222" s="16"/>
+      <x:c r="S222" s="16"/>
+      <x:c r="T222" s="16"/>
     </x:row>
     <x:row r="223">
-      <x:c r="A223" s="28"/>
+      <x:c r="A223" s="30"/>
+      <x:c r="B223" s="16"/>
+      <x:c r="C223" s="16"/>
+      <x:c r="D223" s="16"/>
+      <x:c r="E223" s="16"/>
+      <x:c r="F223" s="16"/>
+      <x:c r="G223" s="16"/>
+      <x:c r="H223" s="16"/>
+      <x:c r="I223" s="16"/>
+      <x:c r="J223" s="16"/>
+      <x:c r="K223" s="16"/>
+      <x:c r="L223" s="16"/>
+      <x:c r="M223" s="16"/>
+      <x:c r="N223" s="16"/>
+      <x:c r="O223" s="16"/>
+      <x:c r="P223" s="16"/>
+      <x:c r="Q223" s="16"/>
+      <x:c r="R223" s="16"/>
+      <x:c r="S223" s="16"/>
+      <x:c r="T223" s="16"/>
     </x:row>
     <x:row r="224">
-      <x:c r="A224" s="28"/>
+      <x:c r="A224" s="30"/>
+      <x:c r="B224" s="16"/>
+      <x:c r="C224" s="16"/>
+      <x:c r="D224" s="16"/>
+      <x:c r="E224" s="16"/>
+      <x:c r="F224" s="16"/>
+      <x:c r="G224" s="16"/>
+      <x:c r="H224" s="16"/>
+      <x:c r="I224" s="16"/>
+      <x:c r="J224" s="16"/>
+      <x:c r="K224" s="16"/>
+      <x:c r="L224" s="16"/>
+      <x:c r="M224" s="16"/>
+      <x:c r="N224" s="16"/>
+      <x:c r="O224" s="16"/>
+      <x:c r="P224" s="16"/>
+      <x:c r="Q224" s="16"/>
+      <x:c r="R224" s="16"/>
+      <x:c r="S224" s="16"/>
+      <x:c r="T224" s="16"/>
     </x:row>
     <x:row r="225">
-      <x:c r="A225" s="28"/>
+      <x:c r="A225" s="30"/>
+      <x:c r="B225" s="16"/>
+      <x:c r="C225" s="16"/>
+      <x:c r="D225" s="16"/>
+      <x:c r="E225" s="16"/>
+      <x:c r="F225" s="16"/>
+      <x:c r="G225" s="16"/>
+      <x:c r="H225" s="16"/>
+      <x:c r="I225" s="16"/>
+      <x:c r="J225" s="16"/>
+      <x:c r="K225" s="16"/>
+      <x:c r="L225" s="16"/>
+      <x:c r="M225" s="16"/>
+      <x:c r="N225" s="16"/>
+      <x:c r="O225" s="16"/>
+      <x:c r="P225" s="16"/>
+      <x:c r="Q225" s="16"/>
+      <x:c r="R225" s="16"/>
+      <x:c r="S225" s="16"/>
+      <x:c r="T225" s="16"/>
     </x:row>
     <x:row r="226">
-      <x:c r="A226" s="28"/>
+      <x:c r="A226" s="30"/>
+      <x:c r="B226" s="16"/>
+      <x:c r="C226" s="16"/>
+      <x:c r="D226" s="16"/>
+      <x:c r="E226" s="16"/>
+      <x:c r="F226" s="16"/>
+      <x:c r="G226" s="16"/>
+      <x:c r="H226" s="16"/>
+      <x:c r="I226" s="16"/>
+      <x:c r="J226" s="16"/>
+      <x:c r="K226" s="16"/>
+      <x:c r="L226" s="16"/>
+      <x:c r="M226" s="16"/>
+      <x:c r="N226" s="16"/>
+      <x:c r="O226" s="16"/>
+      <x:c r="P226" s="16"/>
+      <x:c r="Q226" s="16"/>
+      <x:c r="R226" s="16"/>
+      <x:c r="S226" s="16"/>
+      <x:c r="T226" s="16"/>
     </x:row>
     <x:row r="227">
-      <x:c r="A227" s="28"/>
+      <x:c r="A227" s="30"/>
+      <x:c r="B227" s="16"/>
+      <x:c r="C227" s="16"/>
+      <x:c r="D227" s="16"/>
+      <x:c r="E227" s="16"/>
+      <x:c r="F227" s="16"/>
+      <x:c r="G227" s="16"/>
+      <x:c r="H227" s="16"/>
+      <x:c r="I227" s="16"/>
+      <x:c r="J227" s="16"/>
+      <x:c r="K227" s="16"/>
+      <x:c r="L227" s="16"/>
+      <x:c r="M227" s="16"/>
+      <x:c r="N227" s="16"/>
+      <x:c r="O227" s="16"/>
+      <x:c r="P227" s="16"/>
+      <x:c r="Q227" s="16"/>
+      <x:c r="R227" s="16"/>
+      <x:c r="S227" s="16"/>
+      <x:c r="T227" s="16"/>
     </x:row>
     <x:row r="228">
-      <x:c r="A228" s="28"/>
+      <x:c r="A228" s="30"/>
+      <x:c r="B228" s="16"/>
+      <x:c r="C228" s="16"/>
+      <x:c r="D228" s="16"/>
+      <x:c r="E228" s="16"/>
+      <x:c r="F228" s="16"/>
+      <x:c r="G228" s="16"/>
+      <x:c r="H228" s="16"/>
+      <x:c r="I228" s="16"/>
+      <x:c r="J228" s="16"/>
+      <x:c r="K228" s="16"/>
+      <x:c r="L228" s="16"/>
+      <x:c r="M228" s="16"/>
+      <x:c r="N228" s="16"/>
+      <x:c r="O228" s="16"/>
+      <x:c r="P228" s="16"/>
+      <x:c r="Q228" s="16"/>
+      <x:c r="R228" s="16"/>
+      <x:c r="S228" s="16"/>
+      <x:c r="T228" s="16"/>
     </x:row>
     <x:row r="229">
-      <x:c r="A229" s="28"/>
+      <x:c r="A229" s="30"/>
+      <x:c r="B229" s="16"/>
+      <x:c r="C229" s="16"/>
+      <x:c r="D229" s="16"/>
+      <x:c r="E229" s="16"/>
+      <x:c r="F229" s="16"/>
+      <x:c r="G229" s="16"/>
+      <x:c r="H229" s="16"/>
+      <x:c r="I229" s="16"/>
+      <x:c r="J229" s="16"/>
+      <x:c r="K229" s="16"/>
+      <x:c r="L229" s="16"/>
+      <x:c r="M229" s="16"/>
+      <x:c r="N229" s="16"/>
+      <x:c r="O229" s="16"/>
+      <x:c r="P229" s="16"/>
+      <x:c r="Q229" s="16"/>
+      <x:c r="R229" s="16"/>
+      <x:c r="S229" s="16"/>
+      <x:c r="T229" s="16"/>
     </x:row>
     <x:row r="230">
-      <x:c r="A230" s="28"/>
+      <x:c r="A230" s="30"/>
+      <x:c r="B230" s="16"/>
+      <x:c r="C230" s="16"/>
+      <x:c r="D230" s="16"/>
+      <x:c r="E230" s="16"/>
+      <x:c r="F230" s="16"/>
+      <x:c r="G230" s="16"/>
+      <x:c r="H230" s="16"/>
+      <x:c r="I230" s="16"/>
+      <x:c r="J230" s="16"/>
+      <x:c r="K230" s="16"/>
+      <x:c r="L230" s="16"/>
+      <x:c r="M230" s="16"/>
+      <x:c r="N230" s="16"/>
+      <x:c r="O230" s="16"/>
+      <x:c r="P230" s="16"/>
+      <x:c r="Q230" s="16"/>
+      <x:c r="R230" s="16"/>
+      <x:c r="S230" s="16"/>
+      <x:c r="T230" s="16"/>
     </x:row>
     <x:row r="231">
-      <x:c r="A231" s="28"/>
+      <x:c r="A231" s="30"/>
+      <x:c r="B231" s="16"/>
+      <x:c r="C231" s="16"/>
+      <x:c r="D231" s="16"/>
+      <x:c r="E231" s="16"/>
+      <x:c r="F231" s="16"/>
+      <x:c r="G231" s="16"/>
+      <x:c r="H231" s="16"/>
+      <x:c r="I231" s="16"/>
+      <x:c r="J231" s="16"/>
+      <x:c r="K231" s="16"/>
+      <x:c r="L231" s="16"/>
+      <x:c r="M231" s="16"/>
+      <x:c r="N231" s="16"/>
+      <x:c r="O231" s="16"/>
+      <x:c r="P231" s="16"/>
+      <x:c r="Q231" s="16"/>
+      <x:c r="R231" s="16"/>
+      <x:c r="S231" s="16"/>
+      <x:c r="T231" s="16"/>
     </x:row>
     <x:row r="232">
-      <x:c r="A232" s="28"/>
+      <x:c r="A232" s="30"/>
+      <x:c r="B232" s="16"/>
+      <x:c r="C232" s="16"/>
+      <x:c r="D232" s="16"/>
+      <x:c r="E232" s="16"/>
+      <x:c r="F232" s="16"/>
+      <x:c r="G232" s="16"/>
+      <x:c r="H232" s="16"/>
+      <x:c r="I232" s="16"/>
+      <x:c r="J232" s="16"/>
+      <x:c r="K232" s="16"/>
+      <x:c r="L232" s="16"/>
+      <x:c r="M232" s="16"/>
+      <x:c r="N232" s="16"/>
+      <x:c r="O232" s="16"/>
+      <x:c r="P232" s="16"/>
+      <x:c r="Q232" s="16"/>
+      <x:c r="R232" s="16"/>
+      <x:c r="S232" s="16"/>
+      <x:c r="T232" s="16"/>
     </x:row>
     <x:row r="233">
-      <x:c r="A233" s="28"/>
+      <x:c r="A233" s="30"/>
+      <x:c r="B233" s="16"/>
+      <x:c r="C233" s="16"/>
+      <x:c r="D233" s="16"/>
+      <x:c r="E233" s="16"/>
+      <x:c r="F233" s="16"/>
+      <x:c r="G233" s="16"/>
+      <x:c r="H233" s="16"/>
+      <x:c r="I233" s="16"/>
+      <x:c r="J233" s="16"/>
+      <x:c r="K233" s="16"/>
+      <x:c r="L233" s="16"/>
+      <x:c r="M233" s="16"/>
+      <x:c r="N233" s="16"/>
+      <x:c r="O233" s="16"/>
+      <x:c r="P233" s="16"/>
+      <x:c r="Q233" s="16"/>
+      <x:c r="R233" s="16"/>
+      <x:c r="S233" s="16"/>
+      <x:c r="T233" s="16"/>
     </x:row>
     <x:row r="234">
-      <x:c r="A234" s="28"/>
+      <x:c r="A234" s="30"/>
+      <x:c r="B234" s="16"/>
+      <x:c r="C234" s="16"/>
+      <x:c r="D234" s="16"/>
+      <x:c r="E234" s="16"/>
+      <x:c r="F234" s="16"/>
+      <x:c r="G234" s="16"/>
+      <x:c r="H234" s="16"/>
+      <x:c r="I234" s="16"/>
+      <x:c r="J234" s="16"/>
+      <x:c r="K234" s="16"/>
+      <x:c r="L234" s="16"/>
+      <x:c r="M234" s="16"/>
+      <x:c r="N234" s="16"/>
+      <x:c r="O234" s="16"/>
+      <x:c r="P234" s="16"/>
+      <x:c r="Q234" s="16"/>
+      <x:c r="R234" s="16"/>
+      <x:c r="S234" s="16"/>
+      <x:c r="T234" s="16"/>
     </x:row>
     <x:row r="235">
-      <x:c r="A235" s="28"/>
+      <x:c r="A235" s="30"/>
+      <x:c r="B235" s="16"/>
+      <x:c r="C235" s="16"/>
+      <x:c r="D235" s="16"/>
+      <x:c r="E235" s="16"/>
+      <x:c r="F235" s="16"/>
+      <x:c r="G235" s="16"/>
+      <x:c r="H235" s="16"/>
+      <x:c r="I235" s="16"/>
+      <x:c r="J235" s="16"/>
+      <x:c r="K235" s="16"/>
+      <x:c r="L235" s="16"/>
+      <x:c r="M235" s="16"/>
+      <x:c r="N235" s="16"/>
+      <x:c r="O235" s="16"/>
+      <x:c r="P235" s="16"/>
+      <x:c r="Q235" s="16"/>
+      <x:c r="R235" s="16"/>
+      <x:c r="S235" s="16"/>
+      <x:c r="T235" s="16"/>
     </x:row>
     <x:row r="236">
-      <x:c r="A236" s="28"/>
+      <x:c r="A236" s="30"/>
+      <x:c r="B236" s="16"/>
+      <x:c r="C236" s="16"/>
+      <x:c r="D236" s="16"/>
+      <x:c r="E236" s="16"/>
+      <x:c r="F236" s="16"/>
+      <x:c r="G236" s="16"/>
+      <x:c r="H236" s="16"/>
+      <x:c r="I236" s="16"/>
+      <x:c r="J236" s="16"/>
+      <x:c r="K236" s="16"/>
+      <x:c r="L236" s="16"/>
+      <x:c r="M236" s="16"/>
+      <x:c r="N236" s="16"/>
+      <x:c r="O236" s="16"/>
+      <x:c r="P236" s="16"/>
+      <x:c r="Q236" s="16"/>
+      <x:c r="R236" s="16"/>
+      <x:c r="S236" s="16"/>
+      <x:c r="T236" s="16"/>
     </x:row>
     <x:row r="237">
-      <x:c r="A237" s="28"/>
+      <x:c r="A237" s="30"/>
+      <x:c r="B237" s="16"/>
+      <x:c r="C237" s="16"/>
+      <x:c r="D237" s="16"/>
+      <x:c r="E237" s="16"/>
+      <x:c r="F237" s="16"/>
+      <x:c r="G237" s="16"/>
+      <x:c r="H237" s="16"/>
+      <x:c r="I237" s="16"/>
+      <x:c r="J237" s="16"/>
+      <x:c r="K237" s="16"/>
+      <x:c r="L237" s="16"/>
+      <x:c r="M237" s="16"/>
+      <x:c r="N237" s="16"/>
+      <x:c r="O237" s="16"/>
+      <x:c r="P237" s="16"/>
+      <x:c r="Q237" s="16"/>
+      <x:c r="R237" s="16"/>
+      <x:c r="S237" s="16"/>
+      <x:c r="T237" s="16"/>
     </x:row>
     <x:row r="238">
-      <x:c r="A238" s="28"/>
+      <x:c r="A238" s="30"/>
+      <x:c r="B238" s="16"/>
+      <x:c r="C238" s="16"/>
+      <x:c r="D238" s="16"/>
+      <x:c r="E238" s="16"/>
+      <x:c r="F238" s="16"/>
+      <x:c r="G238" s="16"/>
+      <x:c r="H238" s="16"/>
+      <x:c r="I238" s="16"/>
+      <x:c r="J238" s="16"/>
+      <x:c r="K238" s="16"/>
+      <x:c r="L238" s="16"/>
+      <x:c r="M238" s="16"/>
+      <x:c r="N238" s="16"/>
+      <x:c r="O238" s="16"/>
+      <x:c r="P238" s="16"/>
+      <x:c r="Q238" s="16"/>
+      <x:c r="R238" s="16"/>
+      <x:c r="S238" s="16"/>
+      <x:c r="T238" s="16"/>
     </x:row>
     <x:row r="239">
-      <x:c r="A239" s="28"/>
+      <x:c r="A239" s="30"/>
+      <x:c r="B239" s="16"/>
+      <x:c r="C239" s="16"/>
+      <x:c r="D239" s="16"/>
+      <x:c r="E239" s="16"/>
+      <x:c r="F239" s="16"/>
+      <x:c r="G239" s="16"/>
+      <x:c r="H239" s="16"/>
+      <x:c r="I239" s="16"/>
+      <x:c r="J239" s="16"/>
+      <x:c r="K239" s="16"/>
+      <x:c r="L239" s="16"/>
+      <x:c r="M239" s="16"/>
+      <x:c r="N239" s="16"/>
+      <x:c r="O239" s="16"/>
+      <x:c r="P239" s="16"/>
+      <x:c r="Q239" s="16"/>
+      <x:c r="R239" s="16"/>
+      <x:c r="S239" s="16"/>
+      <x:c r="T239" s="16"/>
     </x:row>
     <x:row r="240">
-      <x:c r="A240" s="28"/>
+      <x:c r="A240" s="30"/>
+      <x:c r="B240" s="16"/>
+      <x:c r="C240" s="16"/>
+      <x:c r="D240" s="16"/>
+      <x:c r="E240" s="16"/>
+      <x:c r="F240" s="16"/>
+      <x:c r="G240" s="16"/>
+      <x:c r="H240" s="16"/>
+      <x:c r="I240" s="16"/>
+      <x:c r="J240" s="16"/>
+      <x:c r="K240" s="16"/>
+      <x:c r="L240" s="16"/>
+      <x:c r="M240" s="16"/>
+      <x:c r="N240" s="16"/>
+      <x:c r="O240" s="16"/>
+      <x:c r="P240" s="16"/>
+      <x:c r="Q240" s="16"/>
+      <x:c r="R240" s="16"/>
+      <x:c r="S240" s="16"/>
+      <x:c r="T240" s="16"/>
     </x:row>
     <x:row r="241">
-      <x:c r="A241" s="28"/>
+      <x:c r="A241" s="30"/>
+      <x:c r="B241" s="16"/>
+      <x:c r="C241" s="16"/>
+      <x:c r="D241" s="16"/>
+      <x:c r="E241" s="16"/>
+      <x:c r="F241" s="16"/>
+      <x:c r="G241" s="16"/>
+      <x:c r="H241" s="16"/>
+      <x:c r="I241" s="16"/>
+      <x:c r="J241" s="16"/>
+      <x:c r="K241" s="16"/>
+      <x:c r="L241" s="16"/>
+      <x:c r="M241" s="16"/>
+      <x:c r="N241" s="16"/>
+      <x:c r="O241" s="16"/>
+      <x:c r="P241" s="16"/>
+      <x:c r="Q241" s="16"/>
+      <x:c r="R241" s="16"/>
+      <x:c r="S241" s="16"/>
+      <x:c r="T241" s="16"/>
     </x:row>
     <x:row r="242">
-      <x:c r="A242" s="28"/>
+      <x:c r="A242" s="30"/>
+      <x:c r="B242" s="16"/>
+      <x:c r="C242" s="16"/>
+      <x:c r="D242" s="16"/>
+      <x:c r="E242" s="16"/>
+      <x:c r="F242" s="16"/>
+      <x:c r="G242" s="16"/>
+      <x:c r="H242" s="16"/>
+      <x:c r="I242" s="16"/>
+      <x:c r="J242" s="16"/>
+      <x:c r="K242" s="16"/>
+      <x:c r="L242" s="16"/>
+      <x:c r="M242" s="16"/>
+      <x:c r="N242" s="16"/>
+      <x:c r="O242" s="16"/>
+      <x:c r="P242" s="16"/>
+      <x:c r="Q242" s="16"/>
+      <x:c r="R242" s="16"/>
+      <x:c r="S242" s="16"/>
+      <x:c r="T242" s="16"/>
     </x:row>
     <x:row r="243">
-      <x:c r="A243" s="28"/>
+      <x:c r="A243" s="30"/>
+      <x:c r="B243" s="16"/>
+      <x:c r="C243" s="16"/>
+      <x:c r="D243" s="16"/>
+      <x:c r="E243" s="16"/>
+      <x:c r="F243" s="16"/>
+      <x:c r="G243" s="16"/>
+      <x:c r="H243" s="16"/>
+      <x:c r="I243" s="16"/>
+      <x:c r="J243" s="16"/>
+      <x:c r="K243" s="16"/>
+      <x:c r="L243" s="16"/>
+      <x:c r="M243" s="16"/>
+      <x:c r="N243" s="16"/>
+      <x:c r="O243" s="16"/>
+      <x:c r="P243" s="16"/>
+      <x:c r="Q243" s="16"/>
+      <x:c r="R243" s="16"/>
+      <x:c r="S243" s="16"/>
+      <x:c r="T243" s="16"/>
     </x:row>
     <x:row r="244">
-      <x:c r="A244" s="28"/>
+      <x:c r="A244" s="30"/>
+      <x:c r="B244" s="16"/>
+      <x:c r="C244" s="16"/>
+      <x:c r="D244" s="16"/>
+      <x:c r="E244" s="16"/>
+      <x:c r="F244" s="16"/>
+      <x:c r="G244" s="16"/>
+      <x:c r="H244" s="16"/>
+      <x:c r="I244" s="16"/>
+      <x:c r="J244" s="16"/>
+      <x:c r="K244" s="16"/>
+      <x:c r="L244" s="16"/>
+      <x:c r="M244" s="16"/>
+      <x:c r="N244" s="16"/>
+      <x:c r="O244" s="16"/>
+      <x:c r="P244" s="16"/>
+      <x:c r="Q244" s="16"/>
+      <x:c r="R244" s="16"/>
+      <x:c r="S244" s="16"/>
+      <x:c r="T244" s="16"/>
     </x:row>
     <x:row r="245">
-      <x:c r="A245" s="28"/>
+      <x:c r="A245" s="30"/>
+      <x:c r="B245" s="16"/>
+      <x:c r="C245" s="16"/>
+      <x:c r="D245" s="16"/>
+      <x:c r="E245" s="16"/>
+      <x:c r="F245" s="16"/>
+      <x:c r="G245" s="16"/>
+      <x:c r="H245" s="16"/>
+      <x:c r="I245" s="16"/>
+      <x:c r="J245" s="16"/>
+      <x:c r="K245" s="16"/>
+      <x:c r="L245" s="16"/>
+      <x:c r="M245" s="16"/>
+      <x:c r="N245" s="16"/>
+      <x:c r="O245" s="16"/>
+      <x:c r="P245" s="16"/>
+      <x:c r="Q245" s="16"/>
+      <x:c r="R245" s="16"/>
+      <x:c r="S245" s="16"/>
+      <x:c r="T245" s="16"/>
     </x:row>
     <x:row r="246">
-      <x:c r="A246" s="28"/>
+      <x:c r="A246" s="30"/>
+      <x:c r="B246" s="16"/>
+      <x:c r="C246" s="16"/>
+      <x:c r="D246" s="16"/>
+      <x:c r="E246" s="16"/>
+      <x:c r="F246" s="16"/>
+      <x:c r="G246" s="16"/>
+      <x:c r="H246" s="16"/>
+      <x:c r="I246" s="16"/>
+      <x:c r="J246" s="16"/>
+      <x:c r="K246" s="16"/>
+      <x:c r="L246" s="16"/>
+      <x:c r="M246" s="16"/>
+      <x:c r="N246" s="16"/>
+      <x:c r="O246" s="16"/>
+      <x:c r="P246" s="16"/>
+      <x:c r="Q246" s="16"/>
+      <x:c r="R246" s="16"/>
+      <x:c r="S246" s="16"/>
+      <x:c r="T246" s="16"/>
     </x:row>
     <x:row r="247">
-      <x:c r="A247" s="28"/>
+      <x:c r="A247" s="30"/>
+      <x:c r="B247" s="16"/>
+      <x:c r="C247" s="16"/>
+      <x:c r="D247" s="16"/>
+      <x:c r="E247" s="16"/>
+      <x:c r="F247" s="16"/>
+      <x:c r="G247" s="16"/>
+      <x:c r="H247" s="16"/>
+      <x:c r="I247" s="16"/>
+      <x:c r="J247" s="16"/>
+      <x:c r="K247" s="16"/>
+      <x:c r="L247" s="16"/>
+      <x:c r="M247" s="16"/>
+      <x:c r="N247" s="16"/>
+      <x:c r="O247" s="16"/>
+      <x:c r="P247" s="16"/>
+      <x:c r="Q247" s="16"/>
+      <x:c r="R247" s="16"/>
+      <x:c r="S247" s="16"/>
+      <x:c r="T247" s="16"/>
     </x:row>
     <x:row r="248">
-      <x:c r="A248" s="28"/>
+      <x:c r="A248" s="30"/>
+      <x:c r="B248" s="16"/>
+      <x:c r="C248" s="16"/>
+      <x:c r="D248" s="16"/>
+      <x:c r="E248" s="16"/>
+      <x:c r="F248" s="16"/>
+      <x:c r="G248" s="16"/>
+      <x:c r="H248" s="16"/>
+      <x:c r="I248" s="16"/>
+      <x:c r="J248" s="16"/>
+      <x:c r="K248" s="16"/>
+      <x:c r="L248" s="16"/>
+      <x:c r="M248" s="16"/>
+      <x:c r="N248" s="16"/>
+      <x:c r="O248" s="16"/>
+      <x:c r="P248" s="16"/>
+      <x:c r="Q248" s="16"/>
+      <x:c r="R248" s="16"/>
+      <x:c r="S248" s="16"/>
+      <x:c r="T248" s="16"/>
     </x:row>
     <x:row r="249">
-      <x:c r="A249" s="28"/>
+      <x:c r="A249" s="30"/>
+      <x:c r="B249" s="16"/>
+      <x:c r="C249" s="16"/>
+      <x:c r="D249" s="16"/>
+      <x:c r="E249" s="16"/>
+      <x:c r="F249" s="16"/>
+      <x:c r="G249" s="16"/>
+      <x:c r="H249" s="16"/>
+      <x:c r="I249" s="16"/>
+      <x:c r="J249" s="16"/>
+      <x:c r="K249" s="16"/>
+      <x:c r="L249" s="16"/>
+      <x:c r="M249" s="16"/>
+      <x:c r="N249" s="16"/>
+      <x:c r="O249" s="16"/>
+      <x:c r="P249" s="16"/>
+      <x:c r="Q249" s="16"/>
+      <x:c r="R249" s="16"/>
+      <x:c r="S249" s="16"/>
+      <x:c r="T249" s="16"/>
     </x:row>
     <x:row r="250">
-      <x:c r="A250" s="28"/>
+      <x:c r="A250" s="30"/>
+      <x:c r="B250" s="16"/>
+      <x:c r="C250" s="16"/>
+      <x:c r="D250" s="16"/>
+      <x:c r="E250" s="16"/>
+      <x:c r="F250" s="16"/>
+      <x:c r="G250" s="16"/>
+      <x:c r="H250" s="16"/>
+      <x:c r="I250" s="16"/>
+      <x:c r="J250" s="16"/>
+      <x:c r="K250" s="16"/>
+      <x:c r="L250" s="16"/>
+      <x:c r="M250" s="16"/>
+      <x:c r="N250" s="16"/>
+      <x:c r="O250" s="16"/>
+      <x:c r="P250" s="16"/>
+      <x:c r="Q250" s="16"/>
+      <x:c r="R250" s="16"/>
+      <x:c r="S250" s="16"/>
+      <x:c r="T250" s="16"/>
     </x:row>
     <x:row r="251">
       <x:c r="A251" s="28"/>
@@ -6007,23 +8486,52 @@
       <x:c r="A1000" s="28"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="H2:H1000">
+  <x:conditionalFormatting sqref="J2:J1000">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>$J2="Grade 5"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="K2:K1000">
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>OR($K2="Deferred",$K2="Refused")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="M2:M1000">
+    <x:cfRule type="expression" dxfId="2" priority="3">
+      <x:formula>OR($M2="Deferred",$M2="Refused")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="P2:P1000">
+    <x:cfRule type="expression" dxfId="3" priority="4">
+      <x:formula>OR($P2="Deferred",$P2="Refused")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="7">
+    <x:dataValidation type="list" sqref="I2:I1000">
       <x:formula1>'Reference Values'!$A$2:$A$3</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I1000">
-      <x:formula1>'Reference Values'!$B$2:$B$4</x:formula1>
+    <x:dataValidation type="list" sqref="J2:J1000">
+      <x:formula1>'Reference Values'!$B$2:$B$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J2:K1000">
-      <x:formula1>'Reference Values'!$C$2:$C$3</x:formula1>
+    <x:dataValidation type="list" sqref="K2:K1000">
+      <x:formula1>'Reference Values'!$C$2:$C$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="L2:L1000">
+    <x:dataValidation type="list" sqref="M2:M1000">
+      <x:formula1>'Reference Values'!$C$2:$C$5</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="O2:O1000">
       <x:formula1>'Reference Values'!$D$2:$D$3</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="P2:P1000">
+      <x:formula1>'Reference Values'!$C$2:$C$5</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="R2:R1000">
+      <x:formula1>'Reference Values'!$E$2:$E$20</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d16d1a5588c450b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75c9c65f5e954f87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6034,8 +8542,11 @@
   <x:cols>
     <x:col min="1" max="1" width="6" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="9.5" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="62" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="8" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="56" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -6046,10 +8557,19 @@
         <x:v>Grade Level</x:v>
       </x:c>
       <x:c r="C1" s="19" t="str">
-        <x:v>Yes / No</x:v>
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="D1" s="19" t="str">
         <x:v>HPV Dose</x:v>
+      </x:c>
+      <x:c r="E1" s="19" t="str">
+        <x:v>Reason Code</x:v>
+      </x:c>
+      <x:c r="F1" s="19" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="G1" s="19" t="str">
+        <x:v>Reason Description</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -6060,10 +8580,19 @@
         <x:v>Grade 1</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Given</x:v>
       </x:c>
       <x:c r="D2" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>01 - Parent/caregiver not home or decision-maker (e.g., spouse) unavailable</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>Parent/caregiver not home or decision-maker (e.g., spouse) unavailable</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6074,15 +8603,218 @@
         <x:v>Grade 4</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>No</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="D3" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="E3" t="str">
+        <x:v>02 - Fear of vaccine side effects</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>Fear of vaccine side effects</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="B4" t="str">
+        <x:v>Grade 5</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Refused</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>03 - Concerns over vaccine safety (e.g., past adverse reaction, Dengvaxia)</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Concerns over vaccine safety (e.g., past adverse reaction, Dengvaxia)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="B5" t="str">
         <x:v>Grade 7</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Not Given</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>04 - Refused extra dose (already completed routine vaccines) [campaign-specific]</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Refused extra dose (already completed routine vaccines) [campaign-specific]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="E6" t="str">
+        <x:v>05 - No time due to work or caregiving; no one to accompany child</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>No time due to work or caregiving; no one to accompany child</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="E7" t="str">
+        <x:v>06 - Belief that vaccine is not effective, low quality, or expired</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Belief that vaccine is not effective, low quality, or expired</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="E8" t="str">
+        <x:v>07 - Belief that child is too young for vaccination</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Belief that child is too young for vaccination</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="E9" t="str">
+        <x:v>08 - Already vaccinated or advised against it by private doctor</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Already vaccinated or advised against it by private doctor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="E10" t="str">
+        <x:v>09 - Religious or personal beliefs not aligned with vaccination</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Religious or personal beliefs not aligned with vaccination</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="E11" t="str">
+        <x:v>10 - Lack of trust in the vaccinator</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Lack of trust in the vaccinator</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="E12" t="str">
+        <x:v>11 - Child was sick, just recovered, or recently discharged from hospital</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Child was sick, just recovered, or recently discharged from hospital</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="E13" t="str">
+        <x:v>12 - Unaware of vaccination schedule/activity</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>Unaware of vaccination schedule/activity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="E14" t="str">
+        <x:v>13 - No health worker visit or vaccine promotion in the area</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>No health worker visit or vaccine promotion in the area</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="E15" t="str">
+        <x:v>14 - Child is visiting, recently moved, or not in target client list</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Child is visiting, recently moved, or not in target client list</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="E16" t="str">
+        <x:v>15 - Too far from site or no transportation (geographical challenges)</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Too far from site or no transportation (geographical challenges)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="E17" t="str">
+        <x:v>16 - Language or communication barrier</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Language or communication barrier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="E18" t="str">
+        <x:v>17 - Caregiver has disability or health condition limiting access</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Caregiver has disability or health condition limiting access</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="E19" t="str">
+        <x:v>18 - Fear of injection</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Fear of injection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="E20" t="str">
+        <x:v>19 - Refused with no reason or Other</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Refused with no reason or Other</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Refactor SBI learner reporting: Remove Grade 5 handling, update documentation, and enhance import management tools
- Updated linelist.py to remove Grade 5 HPV processing and related validations, simplifying the workflow to focus on Grades 1, 4, and 7.
- Revised documentation strings and user-facing messages to reflect changes in the reporting process.
- Introduced import_management.py for admin tools to manage line-list imports, including batch rollbacks and cleanup of manual records.
- Removed references to Grade 5 in various functions and UI components across the application.
- Enhanced data validation and error handling for line-list uploads and reporting.
</commit_message>
<xml_diff>
--- a/programs/sbi/assets/SBI_Linelist_Template.xlsx
+++ b/programs/sbi/assets/SBI_Linelist_Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc63cc805bb804975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line List" sheetId="2" r:id="Rca0924703518437d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="3" r:id="R1ed16a2b43f84554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R38f0088f8b424146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line List" sheetId="2" r:id="R38101906c1fc4a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="3" r:id="R99b67dac1a75446e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +42,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -59,6 +59,21 @@
         <x:fgColor rgb="FFEAF1FB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0033A0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0033A0"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -67,7 +82,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -132,6 +147,19 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -398,10 +426,10 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Abra NIP Dashboard — SBI Learner Reporting Template v5.17</x:v>
-      </x:c>
-      <x:c r="B1" s="5"/>
+      <x:c r="A1" s="35" t="str">
+        <x:v>Abra NIP Dashboard — SBI Learner Line List v5.18</x:v>
+      </x:c>
+      <x:c r="B1" s="35"/>
       <x:c r="C1" s="5"/>
       <x:c r="D1" s="5"/>
       <x:c r="E1" s="5"/>
@@ -409,40 +437,44 @@
       <x:c r="G1" s="5"/>
       <x:c r="H1" s="5"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="12" t="str">
+      <x:c r="A3" s="33" t="str">
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Use one row per learner per activity date. The dashboard calculates VaccTrack counts, regional G1/G4/G5/G7 summaries, deferrals/refusals, and reason totals.</x:v>
+        <x:v>Use one row per learner per activity date. The dashboard calculates the Grade 1, Grade 4 and Grade 7 VaccTrack figures, deferral/refusal counts, and reason totals.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="12" t="str">
+      <x:c r="A4" s="33" t="str">
+        <x:v>Daily workflow</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Use one workbook per RHU per activity date. Encode all schools for that day in the same workbook, then upload it to Step 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="33" t="str">
         <x:v>Grade 1 / Grade 7</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B5" s="16" t="str">
         <x:v>Complete both MR Status and Td Status. Leave HPV fields blank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
+    <x:row r="6">
+      <x:c r="A6" s="33" t="str">
         <x:v>Grade 4 Female</x:v>
       </x:c>
-      <x:c r="B5" s="16" t="str">
+      <x:c r="B6" s="16" t="str">
         <x:v>Set HPV Dose to 1 or 2 and complete HPV Status. Leave MR/Td fields blank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="12" t="str">
-        <x:v>Grade 5 Female</x:v>
-      </x:c>
-      <x:c r="B6" s="16" t="str">
-        <x:v>Use HPV Dose 2 only. Grade 5 is tracked for regional reporting and is NOT sent to VaccTrack.</x:v>
-      </x:c>
-    </x:row>
     <x:row r="7">
-      <x:c r="A7" s="12" t="str">
+      <x:c r="A7" s="33" t="str">
         <x:v>Statuses</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
@@ -450,7 +482,7 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="12" t="str">
+      <x:c r="A8" s="33" t="str">
         <x:v>Deferred / Refused</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
@@ -458,7 +490,7 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="12" t="str">
+      <x:c r="A9" s="33" t="str">
         <x:v>Lot / Batch</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
@@ -466,7 +498,7 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="12" t="str">
+      <x:c r="A10" s="33" t="str">
         <x:v>Revisions</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
@@ -474,7 +506,7 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="12" t="str">
+      <x:c r="A11" s="33" t="str">
         <x:v>Learner ID / LRN</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
@@ -482,7 +514,7 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="12" t="str">
+      <x:c r="A12" s="33" t="str">
         <x:v>Privacy</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
@@ -490,16 +522,16 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="12" t="str">
-        <x:v>Regional clinical fields</x:v>
+      <x:c r="A13" s="33" t="str">
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>Address, date of birth, consent/allergy/sick-today screening remain on the official regional recording form; the dashboard does not collect them because they are not needed for reporting calculations.</x:v>
+        <x:v>This dashboard line list covers Grade 1, Grade 4 and Grade 7 SBI reporting for VaccTrack.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A1:B1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -615,7 +647,7 @@
       <x:c r="G2" s="16" t="str">
         <x:v>JUAN</x:v>
       </x:c>
-      <x:c r="H2" s="16" t="str"/>
+      <x:c r="H2" s="16"/>
       <x:c r="I2" s="16" t="str">
         <x:v>Male</x:v>
       </x:c>
@@ -665,7 +697,7 @@
       <x:c r="G3" s="16" t="str">
         <x:v>MARIA</x:v>
       </x:c>
-      <x:c r="H3" s="16" t="str"/>
+      <x:c r="H3" s="16"/>
       <x:c r="I3" s="16" t="str">
         <x:v>Female</x:v>
       </x:c>
@@ -717,7 +749,7 @@
       <x:c r="G4" s="16" t="str">
         <x:v>ANA</x:v>
       </x:c>
-      <x:c r="H4" s="16" t="str"/>
+      <x:c r="H4" s="16"/>
       <x:c r="I4" s="16" t="str">
         <x:v>Female</x:v>
       </x:c>
@@ -765,7 +797,7 @@
       <x:c r="G5" s="16" t="str">
         <x:v>LIZA</x:v>
       </x:c>
-      <x:c r="H5" s="16" t="str"/>
+      <x:c r="H5" s="16"/>
       <x:c r="I5" s="16" t="str">
         <x:v>Female</x:v>
       </x:c>
@@ -796,98 +828,72 @@
         <x:v>46289</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>000003</x:v>
+        <x:v>000004</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>Sample Elementary School 3</x:v>
+        <x:v>Sample High School</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
-        <x:v>5-A</x:v>
+        <x:v>7-A</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>DUMMY-005</x:v>
+        <x:v>DUMMY-006</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>GARCIA</x:v>
+        <x:v>FLORES</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>MIA</x:v>
-      </x:c>
-      <x:c r="H6" s="16" t="str"/>
+        <x:v>PEDRO</x:v>
+      </x:c>
+      <x:c r="H6" s="16"/>
       <x:c r="I6" s="16" t="str">
-        <x:v>Female</x:v>
+        <x:v>Male</x:v>
       </x:c>
       <x:c r="J6" s="16" t="str">
-        <x:v>Grade 5</x:v>
-      </x:c>
-      <x:c r="K6" s="16"/>
-      <x:c r="L6" s="16"/>
-      <x:c r="M6" s="16"/>
-      <x:c r="N6" s="16"/>
-      <x:c r="O6" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="P6" s="16" t="str">
-        <x:v>Not Given</x:v>
-      </x:c>
+        <x:v>Grade 7</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="L6" s="16" t="str">
+        <x:v>MR-LOT-02</x:v>
+      </x:c>
+      <x:c r="M6" s="16" t="str">
+        <x:v>Given</x:v>
+      </x:c>
+      <x:c r="N6" s="16" t="str">
+        <x:v>TD-LOT-02</x:v>
+      </x:c>
+      <x:c r="O6" s="16"/>
+      <x:c r="P6" s="16"/>
       <x:c r="Q6" s="16"/>
       <x:c r="R6" s="16"/>
-      <x:c r="S6" s="16" t="str">
-        <x:v>Identified without HPV Dose 2</x:v>
-      </x:c>
+      <x:c r="S6" s="16"/>
       <x:c r="T6" s="16" t="str">
-        <x:v>DUMMY RECORD - regional tracking only</x:v>
+        <x:v>DUMMY RECORD - delete before real use</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="30" t="n">
-        <x:v>46289</x:v>
-      </x:c>
-      <x:c r="B7" s="16" t="str">
-        <x:v>000004</x:v>
-      </x:c>
-      <x:c r="C7" s="16" t="str">
-        <x:v>Sample High School</x:v>
-      </x:c>
-      <x:c r="D7" s="16" t="str">
-        <x:v>7-A</x:v>
-      </x:c>
-      <x:c r="E7" s="16" t="str">
-        <x:v>DUMMY-006</x:v>
-      </x:c>
-      <x:c r="F7" s="16" t="str">
-        <x:v>FLORES</x:v>
-      </x:c>
-      <x:c r="G7" s="16" t="str">
-        <x:v>PEDRO</x:v>
-      </x:c>
-      <x:c r="H7" s="16" t="str"/>
-      <x:c r="I7" s="16" t="str">
-        <x:v>Male</x:v>
-      </x:c>
-      <x:c r="J7" s="16" t="str">
-        <x:v>Grade 7</x:v>
-      </x:c>
-      <x:c r="K7" s="16" t="str">
-        <x:v>Given</x:v>
-      </x:c>
-      <x:c r="L7" s="16" t="str">
-        <x:v>MR-LOT-02</x:v>
-      </x:c>
-      <x:c r="M7" s="16" t="str">
-        <x:v>Given</x:v>
-      </x:c>
-      <x:c r="N7" s="16" t="str">
-        <x:v>TD-LOT-02</x:v>
-      </x:c>
+      <x:c r="A7" s="30"/>
+      <x:c r="B7" s="16"/>
+      <x:c r="C7" s="16"/>
+      <x:c r="D7" s="16"/>
+      <x:c r="E7" s="16"/>
+      <x:c r="F7" s="16"/>
+      <x:c r="G7" s="16"/>
+      <x:c r="H7" s="16"/>
+      <x:c r="I7" s="16"/>
+      <x:c r="J7" s="16"/>
+      <x:c r="K7" s="16"/>
+      <x:c r="L7" s="16"/>
+      <x:c r="M7" s="16"/>
+      <x:c r="N7" s="16"/>
       <x:c r="O7" s="16"/>
       <x:c r="P7" s="16"/>
       <x:c r="Q7" s="16"/>
       <x:c r="R7" s="16"/>
       <x:c r="S7" s="16"/>
-      <x:c r="T7" s="16" t="str">
-        <x:v>DUMMY RECORD - delete before real use</x:v>
-      </x:c>
+      <x:c r="T7" s="16"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="30"/>
@@ -8511,7 +8517,7 @@
       <x:formula1>'Reference Values'!$A$2:$A$3</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J1000">
-      <x:formula1>'Reference Values'!$B$2:$B$5</x:formula1>
+      <x:formula1>'Reference Values'!$B$2:$B$4</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K2:K1000">
       <x:formula1>'Reference Values'!$C$2:$C$5</x:formula1>
@@ -8531,7 +8537,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75c9c65f5e954f87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11108a71b0184ad3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8620,7 +8626,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="B4" t="str">
-        <x:v>Grade 5</x:v>
+        <x:v>Grade 7</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>Refused</x:v>
@@ -8636,9 +8642,7 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="B5" t="str">
-        <x:v>Grade 7</x:v>
-      </x:c>
+      <x:c r="B5"/>
       <x:c r="C5" t="str">
         <x:v>Not Given</x:v>
       </x:c>

</xml_diff>